<commit_message>
Shopify leads: batch 1 partial (auto, baby)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>238</v>
+        <v>180</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>688</v>
+        <v>630</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>11</v>
+        <v>67</v>
       </c>
       <c r="G7" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -775,27 +775,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Made-in-USA cast iron cookware</t>
+          <t>Small batch hot sauce</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Plastic-free household cleaning and laundry products with refills</t>
+          <t>Bean-to-bar chocolate</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lightweight smooth cast iron cookware</t>
+          <t>American-made Jeep and Bronco parts and accessories (grab bars, door handles, mounts)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -805,7 +805,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Modern kitchen tools, knives and cutting boards</t>
+          <t>In-house CNC-made Jeep and Ford Bronco light mounts and accessories</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -815,7 +815,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
+          <t>Ford Bronco and Raptor performance and off-road parts, including in-house USA-made items</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -825,7 +825,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dog harnesses, collars, leashes and bundles</t>
+          <t>USA-made MOLLE panels and interior storage for Toyota 4Runner, Tacoma, Tundra and Sequoia</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -835,7 +835,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>No-pull dog harnesses, collars and leashes</t>
+          <t>Auto detailing products and supplies</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -845,7 +845,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Single-ingredient freeze-dried dog and cat treats</t>
+          <t>USA-made car detailing chemicals</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -855,7 +855,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>USA-made dog training treats in refillable tins and pouches</t>
+          <t>Car detailing soaps, kits and cleaning accessories</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -865,7 +865,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Natural USA-made dog treats and dog food</t>
+          <t>USA-made motorcycle bags (windshield, handlebar, adventure/pannier bags)</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -875,7 +875,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Heavy-duty collars and rope leashes for large dogs</t>
+          <t>Harley-Davidson motorcycle parts, suspension and accessories (retail store + online)</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -885,10 +885,570 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Handmade dolls, woodland animals and doll clothes</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Wooden toys, blocks and baby teethers</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Baby essentials: bandana bibs, knit swaddles, car seat covers</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Baby feeding: suction bowls, plates, spoons</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Organic baby clothing, play gyms and toys</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Natural skincare, self-tanners and body care (made in USA)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Vegan skincare and body care with refill program</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Plant-based haircare and skincare</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Natural skincare and body care</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Vegan, plastic-free makeup (lip, cheek, multi-sticks, Balmies)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Phone cases and device accessories</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Magnetic phone cases, chargers and mounts</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Desk setup and laptop stands</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Crossbody phone cases and accessories</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Camping hammocks and outdoor gear</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ultralight backpacks and hiking gear</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Bicycle components and tools</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Home gym equipment (folding squat racks, benches)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cycling apparel</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Bikepacking bags</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Weightlifting accessories (belts, grips, straps)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Specialty coffee roaster (beans, subscriptions)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Specialty coffee roaster (subscriptions)</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Small batch coffee roaster</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Small batch specialty coffee roaster</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Book-inspired soy candles and gifts for readers</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Handmade candles, soaps and skincare from Texas</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Engagement rings, wedding bands and fine jewelry</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Vintage-inspired mechanical watches and straps</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Swiss-made automatic watches and straps</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Made-in-USA cast iron cookware</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Plastic-free household cleaning and laundry products with refills</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Lightweight smooth cast iron cookware</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Modern kitchen tools, knives and cutting boards</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Dog harnesses, collars, leashes and bundles</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>No-pull dog harnesses, collars and leashes</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Single-ingredient freeze-dried dog and cat treats</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>USA-made dog training treats in refillable tins and pouches</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Natural USA-made dog treats and dog food</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Heavy-duty collars and rope leashes for large dogs</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>California-made dog collars, leashes and accessories</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Herbal and leaf teas</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Supplements, herbal teas and gummies</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Natural body scrubs, gift sets (self-care)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
         <v>1</v>
       </c>
     </row>
@@ -903,7 +1463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -928,37 +1488,77 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Subscription / repeat-order workflows</t>
+          <t>Bundle/kit inventory sync</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bundle/kit inventory sync</t>
+          <t>Subscription / repeat-order workflows</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Supplier restock notifications</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Pre-order / launch / drop stock management</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B8" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Order status / fulfilment notifications</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -972,7 +1572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -993,120 +1593,400 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>US location not stated in search snippets (only an 843 phone number)</t>
+          <t>missing personalized_email_body</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>likely mid-size/well-known brand</t>
+          <t>missing personalized_subject</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>no decision maker verified.</t>
+          <t>missing personalized_store_observation</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>missing inventory_order_automation_opportunity</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>missing personalized_store_observation</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>missing inventory_order_automation_opportunity</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>No verified product/collection detail and no US location statement in results (8</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>email draft is generic and must be personalised before use.</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>US location not verified in search results</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>email is a Gmail address (listed on own policy pages).</t>
+          <t xml:space="preserve">no specific product/collection detail verified (search budget exhausted). Email </t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>email not written.</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>contact_source_url approximate (email page not pinned in results)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>confirm.</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>US location (Minnesota) only from third-party aggregator (discovery.patsnap.com/</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>not seen stated on own site in results. Email seen in snippet from coloredorgani</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>US base (Beaverton/Portland, Oregon) and founder name only from third-party CB I</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>own site about page does not name founder in results. Verify location and founde</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>US base not confirmed in results (only a hint of Utah connection in NetSuite blo</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>US location not confirmed</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>no specific product/collection detail verified (search budget exhausted)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>also a K-beauty retailer rather than own brand.</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>US base (Santa Barbara, CA) only seen on Wikipedia, not on own site</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>no specific product with variants verified</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Shopify evidence is URL structure only (/pages/)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>a second address support@nomadgoods.com also appears on a gift card page</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>mid-size brand. Email not written.</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>US base not explicitly stated in results (only 'Mon-Fri 9am-5pm EST' hours and U</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No public email found in search results (site refers to a Support page). Strong </t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>find email on support/contact page.</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>email body N words (need 75–120)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Shopify URL structure, US location (Crown Point, Indiana) and email verified</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Shopify URL structure, US location (Austin, Texas) and email verified</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>No public email found in search results (contact page exists but address not sho</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No public email found in search results (contact section only lists text number </t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>no email drafted.</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>US location not stated in search snippets (only an 843 phone number)</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>likely mid-size/well-known brand</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>no decision maker verified.</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1146,7 +2026,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -1156,7 +2036,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -1166,7 +2046,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shopify leads: batch 1 partial (wellness, home, food, jewelry, electronics)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="G2" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>630</v>
+        <v>623</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="G7" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Camping hammocks and outdoor gear</t>
+          <t>Organic cotton women's activewear, made in Los Angeles</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Ultralight backpacks and hiking gear</t>
+          <t>Handmade infant &amp; toddler moccasins and accessories (Texas)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bicycle components and tools</t>
+          <t>Brazilian bikinis designed in California</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Home gym equipment (folding squat racks, benches)</t>
+          <t>Handmade formalwear and accessories for baby boys (Phoenix, AZ)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cycling apparel</t>
+          <t>Women's activewear and swimwear made in Los Angeles</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Bikepacking bags</t>
+          <t>Women's activewear (leggings, sports bras)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Weightlifting accessories (belts, grips, straps)</t>
+          <t>Kettlebells and strength equipment</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Specialty coffee roaster (beans, subscriptions)</t>
+          <t>Camping hammocks and outdoor gear</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Specialty coffee roaster (subscriptions)</t>
+          <t>Ultralight backpacks and hiking gear</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Small batch coffee roaster</t>
+          <t>Bicycle components and tools</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Small batch specialty coffee roaster</t>
+          <t>Home gym equipment (folding squat racks, benches)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
+          <t>Cycling apparel</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
+          <t>Bikepacking bags</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Book-inspired soy candles and gifts for readers</t>
+          <t>Weightlifting accessories (belts, grips, straps)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
+          <t>Specialty coffee roaster (beans, subscriptions)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
+          <t>Specialty coffee roaster (subscriptions)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
+          <t>Small batch coffee roaster</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
+          <t>Small batch specialty coffee roaster</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Handmade candles, soaps and skincare from Texas</t>
+          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
+          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Engagement rings, wedding bands and fine jewelry</t>
+          <t>Book-inspired soy candles and gifts for readers</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vintage-inspired mechanical watches and straps</t>
+          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Swiss-made automatic watches and straps</t>
+          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
+          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
+          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
+          <t>Handmade candles, soaps and skincare from Texas</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Made-in-USA cast iron cookware</t>
+          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Plastic-free household cleaning and laundry products with refills</t>
+          <t>Engagement rings, wedding bands and fine jewelry</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Lightweight smooth cast iron cookware</t>
+          <t>Vintage-inspired mechanical watches and straps</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Modern kitchen tools, knives and cutting boards</t>
+          <t>Swiss-made automatic watches and straps</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
+          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Dog harnesses, collars, leashes and bundles</t>
+          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>No-pull dog harnesses, collars and leashes</t>
+          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Single-ingredient freeze-dried dog and cat treats</t>
+          <t>Made-in-USA cast iron cookware</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>USA-made dog training treats in refillable tins and pouches</t>
+          <t>Plastic-free household cleaning and laundry products with refills</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Natural USA-made dog treats and dog food</t>
+          <t>Lightweight smooth cast iron cookware</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Heavy-duty collars and rope leashes for large dogs</t>
+          <t>Modern kitchen tools, knives and cutting boards</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>California-made dog collars, leashes and accessories</t>
+          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
+          <t>Dog harnesses, collars, leashes and bundles</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
+          <t>No-pull dog harnesses, collars and leashes</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Herbal and leaf teas</t>
+          <t>Single-ingredient freeze-dried dog and cat treats</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Supplements, herbal teas and gummies</t>
+          <t>USA-made dog training treats in refillable tins and pouches</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,10 +1445,80 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>Natural USA-made dog treats and dog food</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Heavy-duty collars and rope leashes for large dogs</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>California-made dog collars, leashes and accessories</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Herbal and leaf teas</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Supplements, herbal teas and gummies</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
           <t>Natural body scrubs, gift sets (self-care)</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="B76" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1488,7 +1558,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3">
@@ -1498,7 +1568,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -1508,7 +1578,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -1597,7 +1667,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -1607,7 +1677,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -1617,7 +1687,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
@@ -1627,23 +1697,23 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1653,31 +1723,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
@@ -1703,7 +1773,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">no specific product/collection detail verified (search budget exhausted). Email </t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1713,7 +1783,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>email not written.</t>
+          <t xml:space="preserve">no specific product/collection detail verified (search budget exhausted). Email </t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1723,17 +1793,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>contact_source_url approximate (email page not pinned in results)</t>
+          <t>email not written.</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>confirm.</t>
+          <t>contact_source_url approximate (email page not pinned in results)</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1743,7 +1813,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>US location (Minnesota) only from third-party aggregator (discovery.patsnap.com/</t>
+          <t>confirm.</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1753,7 +1823,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>not seen stated on own site in results. Email seen in snippet from coloredorgani</t>
+          <t>US location (Minnesota) only from third-party aggregator (discovery.patsnap.com/</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1763,7 +1833,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>US base (Beaverton/Portland, Oregon) and founder name only from third-party CB I</t>
+          <t>not seen stated on own site in results. Email seen in snippet from coloredorgani</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1773,7 +1843,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>own site about page does not name founder in results. Verify location and founde</t>
+          <t>US base (Beaverton/Portland, Oregon) and founder name only from third-party CB I</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1783,7 +1853,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>US base not confirmed in results (only a hint of Utah connection in NetSuite blo</t>
+          <t>own site about page does not name founder in results. Verify location and founde</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1793,7 +1863,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>US location not confirmed</t>
+          <t>US base not confirmed in results (only a hint of Utah connection in NetSuite blo</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1803,7 +1873,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>no specific product/collection detail verified (search budget exhausted)</t>
+          <t>US location not confirmed</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1813,7 +1883,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>also a K-beauty retailer rather than own brand.</t>
+          <t>no specific product/collection detail verified (search budget exhausted)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1823,7 +1893,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>US base (Santa Barbara, CA) only seen on Wikipedia, not on own site</t>
+          <t>also a K-beauty retailer rather than own brand.</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1833,7 +1903,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>no specific product with variants verified</t>
+          <t>US base (Santa Barbara, CA) only seen on Wikipedia, not on own site</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1843,7 +1913,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Shopify evidence is URL structure only (/pages/)</t>
+          <t>no specific product with variants verified</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1853,7 +1923,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>a second address support@nomadgoods.com also appears on a gift card page</t>
+          <t>Shopify evidence is URL structure only (/pages/)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1863,7 +1933,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>mid-size brand. Email not written.</t>
+          <t>a second address support@nomadgoods.com also appears on a gift card page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1873,7 +1943,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>US base not explicitly stated in results (only 'Mon-Fri 9am-5pm EST' hours and U</t>
+          <t>mid-size brand. Email not written.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1883,7 +1953,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">No public email found in search results (site refers to a Support page). Strong </t>
+          <t>US base not explicitly stated in results (only 'Mon-Fri 9am-5pm EST' hours and U</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1893,7 +1963,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>find email on support/contact page.</t>
+          <t xml:space="preserve">No public email found in search results (site refers to a Support page). Strong </t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1903,7 +1973,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>find email on support/contact page.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1913,7 +1983,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Shopify URL structure, US location (Crown Point, Indiana) and email verified</t>
+          <t>Email is the brand's own Gmail shown on product pages (sizing questions)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1923,7 +1993,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Shopify URL structure, US location (Austin, Texas) and email verified</t>
+          <t>Florida studio stated on About Us page</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1933,7 +2003,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>No public email found in search results (contact page exists but address not sho</t>
+          <t>owner not named.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1943,7 +2013,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">No public email found in search results (contact section only lists text number </t>
+          <t>Owners named on About Us page</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1953,7 +2023,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>contact address is a brand Gmail inbox.</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1963,7 +2033,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>US location not stated in search snippets (only an 843 phone number)</t>
+          <t>No specific product/collection detail verified (search budget exhausted)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1973,7 +2043,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>likely mid-size/well-known brand</t>
+          <t>Shopify evidence only /pages/ URL</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1983,7 +2053,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>no decision maker verified.</t>
+          <t>NY location from search summary.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2026,7 +2096,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
@@ -2036,7 +2106,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -2046,7 +2116,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shopify leads: batch 1 partial (fitness)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10">
@@ -600,19 +600,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G2" t="n">
         <v>27</v>
@@ -725,19 +725,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>623</v>
+        <v>615</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="G7" t="n">
         <v>27</v>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Organic cotton women's activewear, made in Los Angeles</t>
+          <t>Womenswear dresses made in New York (organic/linen)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Handmade infant &amp; toddler moccasins and accessories (Texas)</t>
+          <t>Sustainable women's and kids' clothing made in San Diego</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Brazilian bikinis designed in California</t>
+          <t>Vintage-inspired menswear basics and denim (Los Angeles)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Handmade formalwear and accessories for baby boys (Phoenix, AZ)</t>
+          <t>Techwear apparel (Los Angeles)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Women's activewear and swimwear made in Los Angeles</t>
+          <t>Men's and women's denim and outerwear (Los Angeles)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Women's activewear (leggings, sports bras)</t>
+          <t>Petite womenswear (New York)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kettlebells and strength equipment</t>
+          <t>Women's young contemporary clothing boutique (Austin, Texas)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Camping hammocks and outdoor gear</t>
+          <t>Women's fashion: in-house collection plus curated female-founded brands (San Francisco)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ultralight backpacks and hiking gear</t>
+          <t>Organic cotton women's activewear, made in Los Angeles</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Bicycle components and tools</t>
+          <t>Handmade infant &amp; toddler moccasins and accessories (Texas)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Home gym equipment (folding squat racks, benches)</t>
+          <t>Brazilian bikinis designed in California</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cycling apparel</t>
+          <t>Handmade formalwear and accessories for baby boys (Phoenix, AZ)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bikepacking bags</t>
+          <t>Women's activewear and swimwear made in Los Angeles</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Weightlifting accessories (belts, grips, straps)</t>
+          <t>Women's activewear (leggings, sports bras)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Specialty coffee roaster (beans, subscriptions)</t>
+          <t>Kettlebells and strength equipment</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Specialty coffee roaster (subscriptions)</t>
+          <t>Camping hammocks and outdoor gear</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Small batch coffee roaster</t>
+          <t>Ultralight backpacks and hiking gear</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Small batch specialty coffee roaster</t>
+          <t>Bicycle components and tools</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
+          <t>Home gym equipment (folding squat racks, benches)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
+          <t>Cycling apparel</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Book-inspired soy candles and gifts for readers</t>
+          <t>Bikepacking bags</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
+          <t>Weightlifting accessories (belts, grips, straps)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
+          <t>Specialty coffee roaster (beans, subscriptions)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
+          <t>Specialty coffee roaster (subscriptions)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
+          <t>Small batch coffee roaster</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Handmade candles, soaps and skincare from Texas</t>
+          <t>Small batch specialty coffee roaster</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
+          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Engagement rings, wedding bands and fine jewelry</t>
+          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vintage-inspired mechanical watches and straps</t>
+          <t>Book-inspired soy candles and gifts for readers</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Swiss-made automatic watches and straps</t>
+          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
+          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
+          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
+          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Made-in-USA cast iron cookware</t>
+          <t>Handmade candles, soaps and skincare from Texas</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Plastic-free household cleaning and laundry products with refills</t>
+          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Lightweight smooth cast iron cookware</t>
+          <t>Engagement rings, wedding bands and fine jewelry</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Modern kitchen tools, knives and cutting boards</t>
+          <t>Vintage-inspired mechanical watches and straps</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
+          <t>Swiss-made automatic watches and straps</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Dog harnesses, collars, leashes and bundles</t>
+          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>No-pull dog harnesses, collars and leashes</t>
+          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Single-ingredient freeze-dried dog and cat treats</t>
+          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>USA-made dog training treats in refillable tins and pouches</t>
+          <t>Made-in-USA cast iron cookware</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Natural USA-made dog treats and dog food</t>
+          <t>Plastic-free household cleaning and laundry products with refills</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Heavy-duty collars and rope leashes for large dogs</t>
+          <t>Lightweight smooth cast iron cookware</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>California-made dog collars, leashes and accessories</t>
+          <t>Modern kitchen tools, knives and cutting boards</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
+          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
+          <t>Dog harnesses, collars, leashes and bundles</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Herbal and leaf teas</t>
+          <t>No-pull dog harnesses, collars and leashes</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Supplements, herbal teas and gummies</t>
+          <t>Single-ingredient freeze-dried dog and cat treats</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,10 +1515,90 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>USA-made dog training treats in refillable tins and pouches</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Natural USA-made dog treats and dog food</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Heavy-duty collars and rope leashes for large dogs</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>California-made dog collars, leashes and accessories</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Herbal and leaf teas</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Supplements, herbal teas and gummies</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>Natural body scrubs, gift sets (self-care)</t>
         </is>
       </c>
-      <c r="B76" t="n">
+      <c r="B84" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1558,7 +1638,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3">
@@ -1568,7 +1648,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
@@ -1578,7 +1658,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1604,17 +1684,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -2096,7 +2176,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3">
@@ -2106,7 +2186,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -2116,7 +2196,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shopify leads: batch 1 complete (84 US), deliverables + research notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
       </c>
       <c r="F2" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E7" t="n">
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B84"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -775,831 +775,111 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Small batch hot sauce</t>
+          <t>Specialty food and beverage brands</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bean-to-bar chocolate</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>American-made Jeep and Bronco parts and accessories (grab bars, door handles, mounts)</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>In-house CNC-made Jeep and Ford Bronco light mounts and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ford Bronco and Raptor performance and off-road parts, including in-house USA-made items</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>USA-made MOLLE panels and interior storage for Toyota 4Runner, Tacoma, Tundra and Sequoia</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Auto detailing products and supplies</t>
+          <t>Automotive accessories</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>USA-made car detailing chemicals</t>
+          <t>Fashion and clothing brands</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Car detailing soaps, kits and cleaning accessories</t>
+          <t>Electronics and accessories</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>USA-made motorcycle bags (windshield, handlebar, adventure/pannier bags)</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Harley-Davidson motorcycle parts, suspension and accessories (retail store + online)</t>
+          <t>Kitchen and household products</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Handmade dolls, woodland animals and doll clothes</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Wooden toys, blocks and baby teethers</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Baby essentials: bandana bibs, knit swaddles, car seat covers</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Baby feeding: suction bowls, plates, spoons</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Organic baby clothing, play gyms and toys</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Natural skincare, self-tanners and body care (made in USA)</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Vegan skincare and body care with refill program</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Plant-based haircare and skincare</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Natural skincare and body care</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Vegan, plastic-free makeup (lip, cheek, multi-sticks, Balmies)</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Phone cases and device accessories</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Magnetic phone cases, chargers and mounts</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Desk setup and laptop stands</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Crossbody phone cases and accessories</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Womenswear dresses made in New York (organic/linen)</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Sustainable women's and kids' clothing made in San Diego</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Vintage-inspired menswear basics and denim (Los Angeles)</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Techwear apparel (Los Angeles)</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Men's and women's denim and outerwear (Los Angeles)</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Petite womenswear (New York)</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Women's young contemporary clothing boutique (Austin, Texas)</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Women's fashion: in-house collection plus curated female-founded brands (San Francisco)</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Organic cotton women's activewear, made in Los Angeles</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Handmade infant &amp; toddler moccasins and accessories (Texas)</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Brazilian bikinis designed in California</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Handmade formalwear and accessories for baby boys (Phoenix, AZ)</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Women's activewear and swimwear made in Los Angeles</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Women's activewear (leggings, sports bras)</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Kettlebells and strength equipment</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>Camping hammocks and outdoor gear</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Ultralight backpacks and hiking gear</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Bicycle components and tools</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Home gym equipment (folding squat racks, benches)</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Cycling apparel</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Bikepacking bags</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Weightlifting accessories (belts, grips, straps)</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Specialty coffee roaster (beans, subscriptions)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Specialty coffee roaster (subscriptions)</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Small batch coffee roaster</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Small batch specialty coffee roaster</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Craft hot sauce shop (gift sets, small batch sauces)</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Handcrafted solid hardwood furniture (beds, tables, dressers), made to order in the Midwest</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Book-inspired soy candles and gifts for readers</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Handmade pillow covers, inserts and home textiles sewn in a North Carolina studio</t>
-        </is>
-      </c>
-      <c r="B56" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Handcrafted luxury throw pillow covers and USA-filled pillow inserts</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Handmade-to-order colonial and farmhouse lighting (chandeliers, sconces, lanterns) from a Vermont workshop</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Faith-inspired, hand-poured soy/coconut candles from Colorado Springs</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Handmade candles, soaps and skincare from Texas</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Handmade stacking rings and jewelry (gold fill, rose gold fill, sterling, solid 14K)</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Engagement rings, wedding bands and fine jewelry</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Vintage-inspired mechanical watches and straps</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Swiss-made automatic watches and straps</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Solid 14k gold and sterling silver fine jewelry, engagement rings, personalized rings</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Handmade 14k gold fine jewelry, initial and charm pieces</t>
-        </is>
-      </c>
-      <c r="B66" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Fine and personalized jewelry (name rings, signet rings, birthstones)</t>
-        </is>
-      </c>
-      <c r="B67" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Made-in-USA cast iron cookware</t>
-        </is>
-      </c>
-      <c r="B68" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Plastic-free household cleaning and laundry products with refills</t>
-        </is>
-      </c>
-      <c r="B69" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Lightweight smooth cast iron cookware</t>
-        </is>
-      </c>
-      <c r="B70" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Modern kitchen tools, knives and cutting boards</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Non-toxic concentrate cleaning and laundry products with refillable bottles</t>
-        </is>
-      </c>
-      <c r="B72" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Dog harnesses, collars, leashes and bundles</t>
-        </is>
-      </c>
-      <c r="B73" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>No-pull dog harnesses, collars and leashes</t>
-        </is>
-      </c>
-      <c r="B74" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Single-ingredient freeze-dried dog and cat treats</t>
-        </is>
-      </c>
-      <c r="B75" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>USA-made dog training treats in refillable tins and pouches</t>
-        </is>
-      </c>
-      <c r="B76" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Natural USA-made dog treats and dog food</t>
-        </is>
-      </c>
-      <c r="B77" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Heavy-duty collars and rope leashes for large dogs</t>
-        </is>
-      </c>
-      <c r="B78" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>California-made dog collars, leashes and accessories</t>
-        </is>
-      </c>
-      <c r="B79" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Loose leaf wellness teas, gift sets, tea subscription</t>
-        </is>
-      </c>
-      <c r="B80" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Organic loose leaf wellness teas, samplers, subscription box</t>
-        </is>
-      </c>
-      <c r="B81" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Herbal and leaf teas</t>
-        </is>
-      </c>
-      <c r="B82" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Supplements, herbal teas and gummies</t>
-        </is>
-      </c>
-      <c r="B83" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Natural body scrubs, gift sets (self-care)</t>
-        </is>
-      </c>
-      <c r="B84" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1638,7 +918,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
@@ -1833,17 +1113,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2063,7 +1343,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email is the brand's own Gmail shown on product pages (sizing questions)</t>
+          <t>Email page not pinned (seen on shipping/accessibility snippets)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2073,7 +1353,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Florida studio stated on About Us page</t>
+          <t>Email is the brand's own Gmail shown on product pages (sizing questions)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2083,7 +1363,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>owner not named.</t>
+          <t>Florida studio stated on About Us page</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2093,7 +1373,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Owners named on About Us page</t>
+          <t>owner not named.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2103,7 +1383,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>contact address is a brand Gmail inbox.</t>
+          <t>Owners named on About Us page</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2113,7 +1393,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified (search budget exhausted)</t>
+          <t>contact address is a brand Gmail inbox.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2123,7 +1403,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Shopify evidence only /pages/ URL</t>
+          <t>No specific product/collection detail verified (search budget exhausted)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2133,7 +1413,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>NY location from search summary.</t>
+          <t>Shopify evidence only /pages/ URL</t>
         </is>
       </c>
       <c r="B41" t="n">

</xml_diff>

<commit_message>
Shopify leads: batch 2 partial + fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>84</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>81</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>50</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>166</v>
+        <v>69</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>81</v>
+        <v>175</v>
       </c>
       <c r="G2" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>84</v>
+        <v>181</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>616</v>
+        <v>519</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
-        <v>81</v>
+        <v>175</v>
       </c>
       <c r="G7" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,107 +779,287 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Fashion and clothing brands</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Automotive accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Fashion and clothing brands</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Electronics and accessories</t>
+          <t>Kitchen and household products</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Automotive accessories</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kitchen and household products</t>
+          <t>Electronics and accessories</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Organic and heirloom garden seeds and seed kits</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Culturally important open-pollinated seeds from small farms</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Health and wellness products</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Designer colored glassware and tableware</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Pickleball paddles and accessories</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Pickleball paddles and gear</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Handmade leather golf headcovers</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -918,7 +1098,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -928,7 +1108,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -938,7 +1118,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -948,7 +1128,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -958,7 +1138,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7">
@@ -968,7 +1148,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -978,7 +1158,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -988,7 +1168,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1027,7 +1207,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -1037,83 +1217,83 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>missing personalized_store_observation</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>missing inventory_order_automation_opportunity</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>missing inventory_order_automation_opportunity</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>missing personalized_store_observation</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1143,27 +1323,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">no specific product/collection detail verified (search budget exhausted). Email </t>
+          <t>Listed email uses catalenahats.com while the store domain is catalenahatters.com</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>email not written.</t>
+          <t>confirm the inbox is current before sending.</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>contact_source_url approximate (email page not pinned in results)</t>
+          <t>Email only on giveaway-terms page</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1173,7 +1353,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>confirm.</t>
+          <t>confirm a contact page lists it.</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1183,7 +1363,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>US location (Minnesota) only from third-party aggregator (discovery.patsnap.com/</t>
+          <t>No public email found (contact page is a form only)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1193,7 +1373,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>not seen stated on own site in results. Email seen in snippet from coloredorgani</t>
+          <t>US location not confirmed in results.</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1203,7 +1383,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>US base (Beaverton/Portland, Oregon) and founder name only from third-party CB I</t>
+          <t>No public email found in results</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1213,7 +1393,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>own site about page does not name founder in results. Verify location and founde</t>
+          <t>location not confirmed</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1223,7 +1403,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>US base not confirmed in results (only a hint of Utah connection in NetSuite blo</t>
+          <t>Shopify proof by URL structure only.</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1233,7 +1413,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>US location not confirmed</t>
+          <t>Georgia location inferred from phone area code, not stated.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1243,7 +1423,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>no specific product/collection detail verified (search budget exhausted)</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1253,7 +1433,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>also a K-beauty retailer rather than own brand.</t>
+          <t>Miami/US location not confirmed on site text in results (only brand name)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1263,7 +1443,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>US base (Santa Barbara, CA) only seen on Wikipedia, not on own site</t>
+          <t>verify address on contact page.</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1273,7 +1453,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>no specific product with variants verified</t>
+          <t>Store states it is winding down operations (Last 100 page)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1283,7 +1463,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Shopify evidence is URL structure only (/pages/)</t>
+          <t>likely inactive soon, so no email written.</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1293,7 +1473,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>a second address support@nomadgoods.com also appears on a gift card page</t>
+          <t>US location not stated in search results (USD pricing only)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1303,7 +1483,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>mid-size brand. Email not written.</t>
+          <t>two email variants seen (hello@simplestitchesfabricshop.com vs hello@simplestitc</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1313,7 +1493,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>US base not explicitly stated in results (only 'Mon-Fri 9am-5pm EST' hours and U</t>
+          <t>US location not confirmed in results (name suggests Texas, not verified)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1323,7 +1503,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">No public email found in search results (site refers to a Support page). Strong </t>
+          <t>email seen on a product page rather than a contact page.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1333,7 +1513,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>find email on support/contact page.</t>
+          <t>Only public email (astrid@) is listed on the wholesale page as 'for wholesale in</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1343,7 +1523,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email page not pinned (seen on shipping/accessibility snippets)</t>
+          <t>no general inbox found. Exact US state not confirmed (founded in SF Bay Area).</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1353,7 +1533,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Email is the brand's own Gmail shown on product pages (sizing questions)</t>
+          <t>Brand has studios in Halifax (Canada) and Los Angeles</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1363,7 +1543,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Florida studio stated on About Us page</t>
+          <t>US entity 'Dormie Golf Workshop USA Inc' on Shop, but primary base may be Canada</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1373,7 +1553,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>owner not named.</t>
+          <t>Shopify (shop.app) and Rockport, TX location verified</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1383,7 +1563,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Owners named on About Us page</t>
+          <t>no business email found in search results</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1393,7 +1573,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>contact address is a brand Gmail inbox.</t>
+          <t>no specific product page verified.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1403,7 +1583,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified (search budget exhausted)</t>
+          <t>US location not confirmed in search results (brand appears linked to SmarterPaw)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1413,7 +1593,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Shopify evidence only /pages/ URL</t>
+          <t>verify base country before sending.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1456,7 +1636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>34</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -1466,7 +1646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>34</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
@@ -1476,7 +1656,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shopify leads: batch 2 complete + review holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E2" t="n">
         <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G2" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
       </c>
       <c r="F7" t="n">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="G7" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -815,11 +815,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -829,27 +829,27 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -1098,7 +1098,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1128,7 +1128,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -1253,7 +1253,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1263,27 +1263,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>missing personalized_store_observation</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>missing personalized_store_observation</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1293,7 +1293,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1303,17 +1303,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1323,17 +1323,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Listed email uses catalenahats.com while the store domain is catalenahatters.com</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>confirm the inbox is current before sending.</t>
+          <t>Listed email uses catalenahats.com while the store domain is catalenahatters.com</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1343,7 +1343,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Email only on giveaway-terms page</t>
+          <t>confirm the inbox is current before sending.</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1353,7 +1353,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>confirm a contact page lists it.</t>
+          <t>Email only on giveaway-terms page</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1363,7 +1363,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>No public email found (contact page is a form only)</t>
+          <t>confirm a contact page lists it.</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1373,7 +1373,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>US location not confirmed in results.</t>
+          <t>No public email found (contact page is a form only)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1383,7 +1383,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>No public email found in results</t>
+          <t>US location not confirmed in results.</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1393,7 +1393,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>location not confirmed</t>
+          <t>No public email found in results</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1403,7 +1403,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Shopify proof by URL structure only.</t>
+          <t>location not confirmed</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1413,7 +1413,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Georgia location inferred from phone area code, not stated.</t>
+          <t>Shopify proof by URL structure only.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1423,7 +1423,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>placeholder left in email</t>
+          <t>Georgia location inferred from phone area code, not stated.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1433,7 +1433,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Miami/US location not confirmed on site text in results (only brand name)</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1443,7 +1443,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>verify address on contact page.</t>
+          <t>Miami/US location not confirmed on site text in results (only brand name)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1453,7 +1453,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Store states it is winding down operations (Last 100 page)</t>
+          <t>verify address on contact page.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1463,7 +1463,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>likely inactive soon, so no email written.</t>
+          <t>Store states it is winding down operations (Last 100 page)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1473,7 +1473,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>US location not stated in search results (USD pricing only)</t>
+          <t>likely inactive soon, so no email written.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1483,7 +1483,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>two email variants seen (hello@simplestitchesfabricshop.com vs hello@simplestitc</t>
+          <t>US location not stated in search results (USD pricing only)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1493,7 +1493,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>US location not confirmed in results (name suggests Texas, not verified)</t>
+          <t>two email variants seen (hello@simplestitchesfabricshop.com vs hello@simplestitc</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1503,7 +1503,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>email seen on a product page rather than a contact page.</t>
+          <t>US location not confirmed in results (name suggests Texas, not verified)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1513,7 +1513,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Only public email (astrid@) is listed on the wholesale page as 'for wholesale in</t>
+          <t>email seen on a product page rather than a contact page.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1523,7 +1523,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>no general inbox found. Exact US state not confirmed (founded in SF Bay Area).</t>
+          <t>Only public email (astrid@) is listed on the wholesale page as 'for wholesale in</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1533,7 +1533,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Brand has studios in Halifax (Canada) and Los Angeles</t>
+          <t>no general inbox found. Exact US state not confirmed (founded in SF Bay Area).</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1543,7 +1543,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>US entity 'Dormie Golf Workshop USA Inc' on Shop, but primary base may be Canada</t>
+          <t>Brand has studios in Halifax (Canada) and Los Angeles</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1553,7 +1553,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Shopify (shop.app) and Rockport, TX location verified</t>
+          <t>US entity 'Dormie Golf Workshop USA Inc' on Shop, but primary base may be Canada</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1563,7 +1563,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>no business email found in search results</t>
+          <t>Shopify (shop.app) and Rockport, TX location verified</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1573,7 +1573,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>no specific product page verified.</t>
+          <t>no business email found in search results</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1583,7 +1583,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>US location not confirmed in search results (brand appears linked to SmarterPaw)</t>
+          <t>no specific product page verified.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1593,7 +1593,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>verify base country before sending.</t>
+          <t>US base inferred from shipping terms, not stated.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4">
@@ -1656,7 +1656,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UK/CA batch 1 complete + holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>177</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>171</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>43</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>83</v>
+        <v>111</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>98</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>177</v>
+        <v>245</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>523</v>
+        <v>455</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>171</v>
+        <v>235</v>
       </c>
       <c r="G7" t="n">
-        <v>43</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -775,21 +775,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Specialty food and beverage brands</t>
+          <t>Fashion and clothing brands</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Fashion and clothing brands</t>
+          <t>Specialty food and beverage brands</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -799,37 +799,37 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
@@ -879,13 +879,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -895,7 +895,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -905,7 +905,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -915,7 +915,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Health and wellness products</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Health and wellness products</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,10 +1055,40 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>Essential oils and aromatherapy</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B33" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1098,7 +1128,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>92</v>
+        <v>128</v>
       </c>
     </row>
     <row r="3">
@@ -1108,7 +1138,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4">
@@ -1118,7 +1148,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5">
@@ -1128,7 +1158,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -1138,7 +1168,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -1148,7 +1178,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -1158,7 +1188,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -1168,7 +1198,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -1207,7 +1237,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
@@ -1217,47 +1247,47 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>missing inventory_order_automation_opportunity</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>missing inventory_order_automation_opportunity</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>7</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>missing personalized_store_observation</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -1267,43 +1297,43 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>missing personalized_store_observation</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1313,7 +1343,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1323,7 +1353,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1333,37 +1363,37 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Listed email uses catalenahats.com while the store domain is catalenahatters.com</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>confirm the inbox is current before sending.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Email only on giveaway-terms page</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>confirm a contact page lists it.</t>
+          <t>Inbox given for workshop bookings</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1373,7 +1403,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>No public email found (contact page is a form only)</t>
+          <t>city conflicting (Guelph vs Waterdown)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1383,7 +1413,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>US location not confirmed in results.</t>
+          <t>Victoria, BC Shopify store verified, but no public email address found in search</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1393,7 +1423,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>No public email found in results</t>
+          <t>Central Alberta Shopify store, but no public email found (only a Contact Us link</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1403,7 +1433,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>location not confirmed</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1413,7 +1443,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Shopify proof by URL structure only.</t>
+          <t>product detail from shop.app only</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1423,7 +1453,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Georgia location inferred from phone area code, not stated.</t>
+          <t>info@marketcandlecompany.com surfaced in a site-restricted search summary but th</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1433,7 +1463,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>placeholder left in email</t>
+          <t>Info@AmaranthStoneware.com appeared in a site-restricted search summary (pages s</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1443,7 +1473,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Miami/US location not confirmed on site text in results (only brand name)</t>
+          <t>other listed address is Orders.AmaranthStoneware@gmail.com (Gmail, not allowed).</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1453,7 +1483,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>verify address on contact page.</t>
+          <t>Only email is an ISP address (telus.net), not on the store's own domain</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1463,7 +1493,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Store states it is winding down operations (Last 100 page)</t>
+          <t>Canadian base implied ("across Canada", /hello-bc/ page) but no explicit address</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1473,7 +1503,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>likely inactive soon, so no email written.</t>
+          <t>Email source recorded as homepage footer, not pinned page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1483,7 +1513,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>US location not stated in search results (USD pricing only)</t>
+          <t>Email info@redbearoutdoors.ca seen in search results for redbearoutdoors.ca/page</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1493,7 +1523,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>two email variants seen (hello@simplestitchesfabricshop.com vs hello@simplestitc</t>
+          <t>exact page carrying the email not pinned. Verify contact page before sending.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1503,7 +1533,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>US location not confirmed in results (name suggests Texas, not verified)</t>
+          <t>No Shopify evidence found (contact URL /contact-us/ is not Shopify structure)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1513,7 +1543,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>email seen on a product page rather than a contact page.</t>
+          <t>no verified product detail. Search budget exhausted.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1523,7 +1553,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Only public email (astrid@) is listed on the wholesale page as 'for wholesale in</t>
+          <t>Email only seen on login-help page (/auth), not a contact page</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1533,7 +1563,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>no general inbox found. Exact US state not confirmed (founded in SF Bay Area).</t>
+          <t>no specific product/variant detail verified</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1543,7 +1573,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Brand has studios in Halifax (Canada) and Los Angeles</t>
+          <t>mid-size brand. Search budget exhausted.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1553,7 +1583,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>US entity 'Dormie Golf Workshop USA Inc' on Shop, but primary base may be Canada</t>
+          <t>Canadian location inferred (.ca, collection title), not stated</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1563,7 +1593,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Shopify (shop.app) and Rockport, TX location verified</t>
+          <t>Two inboxes on FAQ (bambiboobaby.com vs bambiboobabies.com) - confirm correct on</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1573,7 +1603,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>no business email found in search results</t>
+          <t>UK location inferred (.co.uk, UK delivery), no address</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1583,7 +1613,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>no specific product page verified.</t>
+          <t>No specific named product/collection page verified (detail from homepage descrip</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1593,7 +1623,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>US base inferred from shipping terms, not stated.</t>
+          <t>search budget ran out before checking.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1636,7 +1666,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>94</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
@@ -1646,7 +1676,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>94</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -1656,7 +1686,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>93</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 5 US/UK/CA results + holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>245</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>245</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>235</v>
+        <v>292</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>85</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="E2" t="n">
         <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="G2" t="n">
-        <v>43</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="G3" t="n">
-        <v>29</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>84</v>
+        <v>61</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>16</v>
+        <v>39</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>245</v>
+        <v>302</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>455</v>
+        <v>398</v>
       </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>235</v>
+        <v>292</v>
       </c>
       <c r="G7" t="n">
-        <v>85</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -775,21 +775,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Fashion and clothing brands</t>
+          <t>Specialty food and beverage brands</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Specialty food and beverage brands</t>
+          <t>Fashion and clothing brands</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -809,27 +809,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -879,13 +879,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -895,7 +895,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -905,7 +905,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -915,7 +915,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Health and wellness products</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Health and wellness products</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,10 +1085,40 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Essential oils and aromatherapy</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1128,7 +1158,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>128</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3">
@@ -1138,7 +1168,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
@@ -1148,7 +1178,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5">
@@ -1158,7 +1188,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -1168,37 +1198,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Order status / fulfilment notifications</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Order status / fulfilment notifications</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1237,7 +1267,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -1247,7 +1277,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4">
@@ -1257,203 +1287,203 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>missing personalized_store_observation</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>missing personalized_store_observation</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Gmail inbox</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>email not written.</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Inbox given for workshop bookings</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>city conflicting (Guelph vs Waterdown)</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Victoria, BC Shopify store verified, but no public email address found in search</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Central Alberta Shopify store, but no public email found (only a Contact Us link</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>product detail from shop.app only</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>info@marketcandlecompany.com surfaced in a site-restricted search summary but th</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1463,7 +1493,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Info@AmaranthStoneware.com appeared in a site-restricted search summary (pages s</t>
+          <t>email from homepage snippet</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1473,7 +1503,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>other listed address is Orders.AmaranthStoneware@gmail.com (Gmail, not allowed).</t>
+          <t>Two inboxes on contact page: info@cuchara.ca (listed for wholesale) and admin@cu</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1483,7 +1513,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Only email is an ISP address (telus.net), not on the store's own domain</t>
+          <t>confirm main customer inbox. Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1493,7 +1523,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Canadian base implied ("across Canada", /hello-bc/ page) but no explicit address</t>
+          <t>Toronto location appeared only in a search-result summary (brand name suggests Y</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1503,7 +1533,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Email source recorded as homepage footer, not pinned page</t>
+          <t>confirm a stated Canadian address/based-in on site. Shopify proof is URL structu</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1513,7 +1543,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Email info@redbearoutdoors.ca seen in search results for redbearoutdoors.ca/page</t>
+          <t>Email from homepage footer</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1523,7 +1553,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>exact page carrying the email not pinned. Verify contact page before sending.</t>
+          <t>no dedicated contact page pinned</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1533,7 +1563,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>No Shopify evidence found (contact URL /contact-us/ is not Shopify structure)</t>
+          <t>Email seen on legacy (non-Shopify) page snapshot</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1543,7 +1573,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>no verified product detail. Search budget exhausted.</t>
+          <t xml:space="preserve">current Shopify contact page snippet showed only phone/address. Verify email on </t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1553,7 +1583,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email only seen on login-help page (/auth), not a contact page</t>
+          <t>email not drafted.</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1563,7 +1593,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>no specific product/variant detail verified</t>
+          <t>conflicting address canadianglow.ca@gmail.com on product pages</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1573,7 +1603,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>mid-size brand. Search budget exhausted.</t>
+          <t>Terms list a Delaware US address</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1583,7 +1613,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Canadian location inferred (.ca, collection title), not stated</t>
+          <t>resells third-party brands (possible dropship). Likely disqualify.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1593,7 +1623,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Two inboxes on FAQ (bambiboobaby.com vs bambiboobabies.com) - confirm correct on</t>
+          <t>Shopify proof weak (/product/ URL, not Shopify pattern)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1603,7 +1633,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>UK location inferred (.co.uk, UK delivery), no address</t>
+          <t>Store showed a /password page in results</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1613,7 +1643,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>No specific named product/collection page verified (detail from homepage descrip</t>
+          <t>confirm store is open</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1623,7 +1653,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>search budget ran out before checking.</t>
+          <t>surname/title unverified</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1666,7 +1696,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>133</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3">
@@ -1676,7 +1706,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>134</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4">
@@ -1686,7 +1716,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>132</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Australia batch 1 + UK beauty + holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>302</v>
+        <v>342</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>302</v>
+        <v>342</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>292</v>
+        <v>329</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>144</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>117</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G3" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>302</v>
+        <v>342</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>398</v>
+        <v>358</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="G7" t="n">
-        <v>144</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -809,27 +809,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -879,23 +879,23 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Health and wellness products</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -905,7 +905,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -915,7 +915,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Health and wellness products</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,10 +1115,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B37" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1158,7 +1168,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>156</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3">
@@ -1168,7 +1178,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4">
@@ -1178,7 +1188,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -1188,37 +1198,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Supplier restock notifications</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Order status / fulfilment notifications</t>
+          <t>Supplier restock notifications</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Order status / fulfilment notifications</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -1228,7 +1238,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1267,7 +1277,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3">
@@ -1277,7 +1287,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4">
@@ -1287,7 +1297,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -1297,27 +1307,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -1337,13 +1347,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1353,11 +1363,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
@@ -1397,7 +1407,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -1483,7 +1493,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1493,7 +1503,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>email from homepage snippet</t>
+          <t>city/state not stated in results, only 'Australian made'.</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1503,7 +1513,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Two inboxes on contact page: info@cuchara.ca (listed for wholesale) and admin@cu</t>
+          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1513,7 +1523,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>confirm main customer inbox. Shopify proof is URL structure only.</t>
+          <t>city/state not stated.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1523,7 +1533,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Toronto location appeared only in a search-result summary (brand name suggests Y</t>
+          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1533,7 +1543,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>confirm a stated Canadian address/based-in on site. Shopify proof is URL structu</t>
+          <t>no named product seen.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1543,7 +1553,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Email from homepage footer</t>
+          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1553,7 +1563,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>no dedicated contact page pinned</t>
+          <t>no specific product or city verified.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1563,7 +1573,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Email seen on legacy (non-Shopify) page snapshot</t>
+          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1573,7 +1583,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">current Shopify contact page snippet showed only phone/address. Verify email on </t>
+          <t>product URL uses /product/ (non-Shopify path)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1583,7 +1593,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>email not drafted.</t>
+          <t>city not stated.</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1593,7 +1603,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>conflicting address canadianglow.ca@gmail.com on product pages</t>
+          <t>No named product/collection verified (only brand-level small-batch detail)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1603,7 +1613,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Terms list a Delaware US address</t>
+          <t>julia@ is a named address but Julia's role is unverified.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1613,7 +1623,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>resells third-party brands (possible dropship). Likely disqualify.</t>
+          <t>Email seen in product-page snippets but exact page not pinned down</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1623,7 +1633,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Shopify proof weak (/product/ URL, not Shopify pattern)</t>
+          <t>email domain (sanctclothing.com) differs from store domain.</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1633,7 +1643,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Store showed a /password page in results</t>
+          <t>Multiple inboxes seen (hello@, filippa@, support@, plus a gmail for bespoke phot</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1643,7 +1653,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>confirm store is open</t>
+          <t>exact page for hello@ not pinned down.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1653,7 +1663,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>surname/title unverified</t>
+          <t>Outlook.com inbox</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1696,7 +1706,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>184</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3">
@@ -1706,7 +1716,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>185</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4">
@@ -1716,7 +1726,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>183</v>
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Australia fashion + food batches, holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>342</v>
+        <v>338</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>342</v>
+        <v>338</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="G5" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="E7" t="n">
         <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="G7" t="n">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5">
@@ -1168,7 +1168,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -1198,7 +1198,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -1433,7 +1433,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1443,7 +1443,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1453,7 +1453,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1463,7 +1463,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1473,7 +1473,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1483,7 +1483,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1493,17 +1493,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>city/state not stated in results, only 'Australian made'.</t>
+          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1513,7 +1513,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
+          <t>city/state not stated in results, only 'Australian made'.</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1523,7 +1523,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>city/state not stated.</t>
+          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1533,7 +1533,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
+          <t>city/state not stated.</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1543,7 +1543,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>no named product seen.</t>
+          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1553,7 +1553,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
+          <t>no named product seen.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1563,7 +1563,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>no specific product or city verified.</t>
+          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1573,7 +1573,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
+          <t>no specific product or city verified.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1583,7 +1583,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>product URL uses /product/ (non-Shopify path)</t>
+          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1593,7 +1593,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>city not stated.</t>
+          <t>product URL uses /product/ (non-Shopify path)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1603,7 +1603,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>No named product/collection verified (only brand-level small-batch detail)</t>
+          <t>city not stated.</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1613,7 +1613,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>julia@ is a named address but Julia's role is unverified.</t>
+          <t>Better-known label</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1623,7 +1623,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Email seen in product-page snippets but exact page not pinned down</t>
+          <t>may exceed target size</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1633,7 +1633,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>email domain (sanctclothing.com) differs from store domain.</t>
+          <t>No named product/collection verified (only brand-level small-batch detail)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1643,7 +1643,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Multiple inboxes seen (hello@, filippa@, support@, plus a gmail for bespoke phot</t>
+          <t>julia@ is a named address but Julia's role is unverified.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1653,7 +1653,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>exact page for hello@ not pinned down.</t>
+          <t>Email seen in product-page snippets but exact page not pinned down</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1663,7 +1663,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Outlook.com inbox</t>
+          <t>email domain (sanctclothing.com) differs from store domain.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="3">
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4">
@@ -1726,7 +1726,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US seeds B round 7 + hold; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>338</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>338</v>
+        <v>370</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>325</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>185</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>126</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="G2" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>67</v>
+        <v>77</v>
       </c>
       <c r="G3" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G4" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>338</v>
+        <v>370</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>362</v>
+        <v>330</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>325</v>
+        <v>355</v>
       </c>
       <c r="G7" t="n">
-        <v>185</v>
+        <v>209</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>57</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3">
@@ -789,27 +789,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,10 +1125,60 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1168,7 +1218,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>165</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3">
@@ -1178,7 +1228,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -1188,7 +1238,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -1198,7 +1248,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
@@ -1208,7 +1258,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -1218,27 +1268,27 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Order status / fulfilment notifications</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Order status / fulfilment notifications</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1327,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
@@ -1287,7 +1337,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -1297,7 +1347,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -1307,7 +1357,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -1317,7 +1367,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -1327,7 +1377,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -1337,7 +1387,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1373,7 +1423,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1383,11 +1433,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
@@ -1417,13 +1467,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1433,11 +1483,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1463,7 +1513,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1473,7 +1523,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1483,7 +1533,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1493,7 +1543,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1503,17 +1553,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>city/state not stated in results, only 'Australian made'.</t>
+          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1523,7 +1573,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
+          <t>city/state not stated in results, only 'Australian made'.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1533,7 +1583,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>city/state not stated.</t>
+          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1543,7 +1593,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
+          <t>city/state not stated.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1553,7 +1603,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>no named product seen.</t>
+          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1563,7 +1613,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
+          <t>no named product seen.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1573,7 +1623,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>no specific product or city verified.</t>
+          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1583,7 +1633,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
+          <t>no specific product or city verified.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1593,7 +1643,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>product URL uses /product/ (non-Shopify path)</t>
+          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1603,7 +1653,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>city not stated.</t>
+          <t>product URL uses /product/ (non-Shopify path)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1613,7 +1663,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Better-known label</t>
+          <t>city not stated.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1623,7 +1673,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>may exceed target size</t>
+          <t>Better-known label</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1633,7 +1683,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>No named product/collection verified (only brand-level small-batch detail)</t>
+          <t>may exceed target size</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1643,7 +1693,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>julia@ is a named address but Julia's role is unverified.</t>
+          <t>No named product/collection verified (only brand-level small-batch detail)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1653,7 +1703,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Email seen in product-page snippets but exact page not pinned down</t>
+          <t>julia@ is a named address but Julia's role is unverified.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1663,7 +1713,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>email domain (sanctclothing.com) differs from store domain.</t>
+          <t>Email seen in product-page snippets but exact page not pinned down</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1706,7 +1756,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>210</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3">
@@ -1716,7 +1766,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>212</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4">
@@ -1726,7 +1776,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>209</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Germany batch 1 (beauty, pet/baby, home, fit/tech/gifts) + holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>370</v>
+        <v>395</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>370</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>355</v>
+        <v>377</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>132</v>
+        <v>149</v>
       </c>
     </row>
     <row r="10">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>28</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>370</v>
+        <v>395</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>330</v>
+        <v>305</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>355</v>
+        <v>377</v>
       </c>
       <c r="G7" t="n">
-        <v>209</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3">
@@ -789,27 +789,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,10 +1175,100 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>Handmade leather golf headcovers</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B51" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1218,7 +1308,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3">
@@ -1228,7 +1318,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4">
@@ -1238,7 +1328,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -1248,23 +1338,23 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Supplier restock notifications</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Supplier restock notifications</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1327,7 +1417,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3">
@@ -1337,7 +1427,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
@@ -1347,7 +1437,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5">
@@ -1357,27 +1447,27 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -1387,7 +1477,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1397,7 +1487,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
@@ -1433,7 +1523,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -1443,11 +1533,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>placeholder left in email</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1513,7 +1603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1523,7 +1613,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1533,7 +1623,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1543,7 +1633,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1553,7 +1643,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1563,17 +1653,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>city/state not stated in results, only 'Australian made'.</t>
+          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1583,7 +1673,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
+          <t>city/state not stated in results, only 'Australian made'.</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1593,7 +1683,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>city/state not stated.</t>
+          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1603,7 +1693,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
+          <t>city/state not stated.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1613,7 +1703,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>no named product seen.</t>
+          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1623,7 +1713,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
+          <t>no named product seen.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1633,7 +1723,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>no specific product or city verified.</t>
+          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1643,7 +1733,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
+          <t>no specific product or city verified.</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1653,7 +1743,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>product URL uses /product/ (non-Shopify path)</t>
+          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1663,7 +1753,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>city not stated.</t>
+          <t>product URL uses /product/ (non-Shopify path)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1673,7 +1763,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Better-known label</t>
+          <t>city not stated.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1683,7 +1773,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>may exceed target size</t>
+          <t>Better-known label</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1693,7 +1783,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>No named product/collection verified (only brand-level small-batch detail)</t>
+          <t>may exceed target size</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1703,7 +1793,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>julia@ is a named address but Julia's role is unverified.</t>
+          <t>No named product/collection verified (only brand-level small-batch detail)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1713,7 +1803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Email seen in product-page snippets but exact page not pinned down</t>
+          <t>julia@ is a named address but Julia's role is unverified.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1756,7 +1846,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>236</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3">
@@ -1766,7 +1856,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4">
@@ -1776,7 +1866,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>235</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Germany fashion/food + CA beauty/food rows, holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>377</v>
+        <v>385</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>228</v>
+        <v>243</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="G3" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G6" t="n">
         <v>24</v>
-      </c>
-      <c r="G6" t="n">
-        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="G7" t="n">
-        <v>228</v>
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>180</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3">
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4">
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
@@ -1427,7 +1427,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -1477,7 +1477,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>244</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>246</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>243</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AU round 9 fashion/beauty + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>403</v>
+        <v>417</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>403</v>
+        <v>417</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>385</v>
+        <v>399</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>243</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G3" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G5" t="n">
-        <v>34</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>403</v>
+        <v>417</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>385</v>
+        <v>399</v>
       </c>
       <c r="G7" t="n">
-        <v>243</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="3">
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5">
@@ -1467,7 +1467,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8">
@@ -1487,13 +1487,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1503,7 +1503,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1513,27 +1513,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>placeholder left in email</t>
+          <t>Gmail inbox</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -1543,11 +1543,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Gmail inbox</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -1583,7 +1583,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>Email seen on homepage only</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1593,7 +1593,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1603,7 +1603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1613,7 +1613,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1623,7 +1623,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1633,7 +1633,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1643,7 +1643,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1653,7 +1653,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1663,17 +1663,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Two inboxes on FAQ page (orders@ for shipping/general queries, sales@ for return</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>city/state not stated in results, only 'Australian made'.</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1683,7 +1683,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: soapybutter@gmail.com on contact page vs info@soapybutter.c</t>
+          <t>typo address on privacy page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1693,7 +1693,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>city/state not stated.</t>
+          <t>Avril role unconfirmed</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1703,7 +1703,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Conflicting inboxes: sales@celestialsalts.com.au on contact page vs celestialsal</t>
+          <t xml:space="preserve">Only inbox seen is wholesale@ (wholesale page), not confirmed as the main store </t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1713,7 +1713,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>no named product seen.</t>
+          <t>hello@claremakes.com.au appeared in results from claremakes.com.au (stockists/cu</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1723,7 +1723,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conflicting inboxes (hello@naturdermskincare.com.au, info@naturdermskin.com.au, </t>
+          <t>verify contact_source_url.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1733,7 +1733,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>no specific product or city verified.</t>
+          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1743,7 +1743,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two inboxes on contact page (info@ and care@, with a misspelt christianacua.com </t>
+          <t>older page shows info@)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1753,7 +1753,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>product URL uses /product/ (non-Shopify path)</t>
+          <t>.com email vs .com.au site. Some pages may be old.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1763,7 +1763,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>city not stated.</t>
+          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1773,7 +1773,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Better-known label</t>
+          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1783,7 +1783,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>may exceed target size</t>
+          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1793,7 +1793,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>No named product/collection verified (only brand-level small-batch detail)</t>
+          <t>no specific named product.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1803,7 +1803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>julia@ is a named address but Julia's role is unverified.</t>
+          <t>No Shopify evidence (URLs like /about/candle-fragrances/... suggest a non-Shopif</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>254</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3">
@@ -1856,7 +1856,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>256</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>253</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UK jewellery/outdoor round 10 + hold; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>399</v>
+        <v>405</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>270</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="G2" t="n">
-        <v>66</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G3" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G4" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G5" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="G7" t="n">
-        <v>270</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -855,7 +855,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kitchen and household products</t>
+          <t>Automotive accessories</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -865,11 +865,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Automotive accessories</t>
+          <t>Kitchen and household products</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,10 +1265,20 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B52" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1308,7 +1318,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>186</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3">
@@ -1318,27 +1328,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Subscription / repeat-order workflows</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Subscription / repeat-order workflows</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -1348,7 +1358,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7">
@@ -1417,7 +1427,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3">
@@ -1427,7 +1437,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -1437,7 +1447,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -1457,7 +1467,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -1467,7 +1477,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8">
@@ -1477,7 +1487,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -1527,7 +1537,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -1583,17 +1593,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Email seen on homepage only</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>Email seen on homepage only</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1603,7 +1613,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1613,7 +1623,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1623,7 +1633,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1633,7 +1643,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1643,7 +1653,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>resells other brands</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1653,7 +1663,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1663,7 +1673,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1673,27 +1683,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>typo address on privacy page</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Avril role unconfirmed</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1703,7 +1713,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only inbox seen is wholesale@ (wholesale page), not confirmed as the main store </t>
+          <t>typo address on privacy page</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1713,7 +1723,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>hello@claremakes.com.au appeared in results from claremakes.com.au (stockists/cu</t>
+          <t>Avril role unconfirmed</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1723,7 +1733,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>verify contact_source_url.</t>
+          <t xml:space="preserve">Only inbox seen is wholesale@ (wholesale page), not confirmed as the main store </t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1733,7 +1743,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
+          <t>hello@claremakes.com.au appeared in results from claremakes.com.au (stockists/cu</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1743,7 +1753,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>older page shows info@)</t>
+          <t>verify contact_source_url.</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1753,7 +1763,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>.com email vs .com.au site. Some pages may be old.</t>
+          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1763,7 +1773,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
+          <t>older page shows info@)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1773,7 +1783,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
+          <t>.com email vs .com.au site. Some pages may be old.</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1783,7 +1793,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
+          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1793,7 +1803,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>no specific named product.</t>
+          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1803,7 +1813,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>No Shopify evidence (URLs like /about/candle-fragrances/... suggest a non-Shopif</t>
+          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1846,7 +1856,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3">
@@ -1856,7 +1866,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4">
@@ -1866,7 +1876,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE beauty/home, UK food/pet, AU seeds rows; supersedes + holds
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>423</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>423</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>405</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>294</v>
+        <v>323</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>148</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G3" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G5" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>74</v>
+        <v>57</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="G6" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>423</v>
+        <v>450</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>277</v>
+        <v>250</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>405</v>
+        <v>432</v>
       </c>
       <c r="G7" t="n">
-        <v>294</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Yarn / Wolle &amp; Strickzubehör</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Hundehalsbänder aus Naturleder</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,10 +1275,70 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B58" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1318,7 +1378,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>188</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3">
@@ -1328,7 +1388,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -1338,7 +1398,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
@@ -1348,7 +1408,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
@@ -1358,7 +1418,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1374,17 +1434,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Order status / fulfilment notifications</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Order status / fulfilment notifications</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1427,7 +1487,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -1437,7 +1497,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4">
@@ -1463,21 +1523,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>email domain not the business</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>email domain not the business</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
@@ -1487,7 +1547,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -1497,33 +1557,33 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -1567,7 +1627,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1683,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1633,7 +1693,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1643,7 +1703,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1653,7 +1713,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>resells other brands</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1663,7 +1723,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1673,7 +1733,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>resells other brands</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1683,7 +1743,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1693,7 +1753,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1703,27 +1763,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>typo address on privacy page</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Avril role unconfirmed</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1733,7 +1793,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Only inbox seen is wholesale@ (wholesale page), not confirmed as the main store </t>
+          <t>typo address on privacy page</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1743,7 +1803,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>hello@claremakes.com.au appeared in results from claremakes.com.au (stockists/cu</t>
+          <t>Avril role unconfirmed</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1753,7 +1813,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>verify contact_source_url.</t>
+          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1763,7 +1823,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
+          <t>older page shows info@)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1773,7 +1833,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>older page shows info@)</t>
+          <t>.com email vs .com.au site. Some pages may be old.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1783,7 +1843,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>.com email vs .com.au site. Some pages may be old.</t>
+          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1793,7 +1853,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
+          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1803,7 +1863,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
+          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1813,7 +1873,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
+          <t>no specific named product.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1856,7 +1916,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>273</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3">
@@ -1866,7 +1926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>275</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4">
@@ -1876,7 +1936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>272</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE mixed/gifts + AU beauty rows, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>450</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>432</v>
+        <v>436</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="G5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G7" t="n">
-        <v>323</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5">
@@ -815,17 +815,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13">
@@ -895,7 +895,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Ceramics / tableware</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -905,7 +905,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -915,7 +915,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Yarn / Wolle &amp; Strickzubehör</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3">
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4">
@@ -1398,7 +1398,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -1418,7 +1418,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1633,7 +1633,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>Email seen on homepage only</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1643,7 +1643,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1653,7 +1653,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1663,11 +1663,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Email seen on homepage only</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AU round 12 + DE pet/baby rows, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>436</v>
+        <v>432</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
     <row r="8">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="E5" t="n">
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G5" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>454</v>
+        <v>450</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E7" t="n">
         <v>18</v>
       </c>
       <c r="F7" t="n">
-        <v>436</v>
+        <v>432</v>
       </c>
       <c r="G7" t="n">
-        <v>327</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hundehalsbänder aus Naturleder</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,20 +1325,10 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
-        </is>
-      </c>
-      <c r="B58" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1378,7 +1368,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -1418,7 +1408,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
@@ -1916,7 +1906,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3">
@@ -1926,7 +1916,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4">
@@ -1936,7 +1926,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>294</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US fresh D + UK fashion/fit rows, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>450</v>
+        <v>479</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>450</v>
+        <v>479</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>432</v>
+        <v>459</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>331</v>
+        <v>367</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G2" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="G3" t="n">
-        <v>96</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="G4" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>450</v>
+        <v>479</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>250</v>
+        <v>221</v>
       </c>
       <c r="E7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>432</v>
+        <v>459</v>
       </c>
       <c r="G7" t="n">
-        <v>331</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
@@ -809,17 +809,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
@@ -829,17 +829,17 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Craft supplies / hand-dyed fibre, yarn and knitting kits</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Stationery / undated planners, notebooks and log books</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,10 +1325,40 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1368,7 +1398,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>199</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3">
@@ -1378,7 +1408,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4">
@@ -1388,7 +1418,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5">
@@ -1398,7 +1428,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6">
@@ -1418,7 +1448,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -1428,7 +1458,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -1438,7 +1468,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1477,7 +1507,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>84</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -1487,7 +1517,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>75</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -1497,7 +1527,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
@@ -1507,7 +1537,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -1517,7 +1547,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -1527,67 +1557,67 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>no research source URL</t>
+          <t>Gmail inbox</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Gmail inbox</t>
+          <t>no research source URL</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -1693,7 +1723,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1703,7 +1733,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1713,7 +1743,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1723,7 +1753,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>resells other brands</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1733,7 +1763,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>resells other brands</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1743,7 +1773,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1753,7 +1783,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1763,7 +1793,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1773,27 +1803,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>typo address on privacy page</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Avril role unconfirmed</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1803,7 +1833,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
+          <t>typo address on privacy page</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1813,7 +1843,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>older page shows info@)</t>
+          <t>Avril role unconfirmed</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1823,7 +1853,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>.com email vs .com.au site. Some pages may be old.</t>
+          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1833,7 +1863,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
+          <t>older page shows info@)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1843,7 +1873,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
+          <t>.com email vs .com.au site. Some pages may be old.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1853,7 +1883,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>two inboxes (orders@ on FAQ, info@ on privacy policy)</t>
+          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1863,7 +1893,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>no specific named product.</t>
+          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1906,7 +1936,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>291</v>
+        <v>318</v>
       </c>
     </row>
     <row r="3">
@@ -1916,7 +1946,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>293</v>
+        <v>320</v>
       </c>
     </row>
     <row r="4">
@@ -1926,7 +1956,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>290</v>
+        <v>317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CA dir B, UK food/pet, UK craft rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>479</v>
+        <v>486</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>479</v>
+        <v>486</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>459</v>
+        <v>467</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="G2" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G3" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G4" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F7" t="n">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="G7" t="n">
-        <v>367</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -789,27 +789,27 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Craft supplies / hand-dyed fibre, yarn and knitting kits</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Stationery / undated planners, notebooks and log books</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,30 +1335,10 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
-        </is>
-      </c>
-      <c r="B59" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
-        </is>
-      </c>
-      <c r="B60" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1398,7 +1378,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="3">
@@ -1408,7 +1388,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4">
@@ -1418,7 +1398,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -1438,7 +1418,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -1448,7 +1428,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1468,7 +1448,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1507,7 +1487,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3">
@@ -1517,7 +1497,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -1527,7 +1507,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5">
@@ -1537,7 +1517,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6">
@@ -1567,7 +1547,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9">
@@ -1587,7 +1567,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
@@ -1673,7 +1653,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1683,7 +1663,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1693,17 +1673,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1713,7 +1693,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1723,7 +1703,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1733,7 +1713,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1743,7 +1723,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1753,7 +1733,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1763,7 +1743,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>resells other brands</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1773,7 +1753,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>resells other brands</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1783,7 +1763,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1793,7 +1773,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1936,7 +1916,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>318</v>
+        <v>326</v>
       </c>
     </row>
     <row r="3">
@@ -1946,7 +1926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>320</v>
+        <v>328</v>
       </c>
     </row>
     <row r="4">
@@ -1956,7 +1936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CA dir C rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="8">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G4" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E7" t="n">
         <v>19</v>
       </c>
       <c r="F7" t="n">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="G7" t="n">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -795,7 +795,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -805,17 +805,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -825,11 +825,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3">
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="3">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US cities round 13 + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="8">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G2" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E7" t="n">
         <v>19</v>
       </c>
       <c r="F7" t="n">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="G7" t="n">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>
@@ -789,23 +789,23 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3">
@@ -1428,7 +1428,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -1448,7 +1448,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="3">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE imp B, AU sweep A, AU fashion/home rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>481</v>
+        <v>530</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>481</v>
+        <v>530</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>462</v>
+        <v>509</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>378</v>
+        <v>439</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G2" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G3" t="n">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="G4" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>52</v>
+        <v>69</v>
       </c>
       <c r="G5" t="n">
-        <v>76</v>
+        <v>111</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="G6" t="n">
-        <v>39</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>481</v>
+        <v>530</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>219</v>
+        <v>170</v>
       </c>
       <c r="E7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>462</v>
+        <v>509</v>
       </c>
       <c r="G7" t="n">
-        <v>378</v>
+        <v>439</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B58"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3">
@@ -789,47 +789,47 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10">
@@ -895,27 +895,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ceramics / tableware</t>
+          <t>Kaffee / Kaffeerösterei</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Ceramics / tableware</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Kaffee / Specialty-Kaffeerösterei</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Taschen (Vintage Louis Vuitton)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Taschen (Lederwaren, Rucksäcke, Geldbörsen)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,10 +1335,110 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>Handmade leather golf headcovers</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
-      <c r="B58" t="n">
+      <c r="B68" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1353,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1378,7 +1478,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>212</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3">
@@ -1388,7 +1488,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>102</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -1398,7 +1498,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
@@ -1408,7 +1508,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -1418,7 +1518,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -1428,7 +1528,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -1449,6 +1549,16 @@
       </c>
       <c r="B9" t="n">
         <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Inventory reporting</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1487,7 +1597,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>96</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3">
@@ -1497,7 +1607,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>87</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4">
@@ -1507,7 +1617,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>73</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -1517,7 +1627,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6">
@@ -1527,27 +1637,27 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>missing product_or_collection</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>missing product_or_collection</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>32</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -1557,7 +1667,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -1567,7 +1677,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -1577,7 +1687,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -1587,7 +1697,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13">
@@ -1597,23 +1707,23 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>placeholder left in email</t>
+          <t>email not written.</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>placeholder left in email</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -1623,11 +1733,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>email not written.</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -1637,43 +1747,43 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1683,27 +1793,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>exact contact page not confirmed.</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1713,7 +1823,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1723,7 +1833,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1733,7 +1843,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1743,7 +1853,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>no product detail or stated location found</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1753,7 +1863,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>resells other brands</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1763,7 +1873,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1773,7 +1883,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1783,7 +1893,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1793,7 +1903,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>no specific product detail verified. Email not written.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1803,67 +1913,67 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>typo address on privacy page</t>
+          <t>Owner name inferred from brand name/inbox</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Avril role unconfirmed</t>
+          <t>resells other brands</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Multiple inboxes (sales@ and advice@fourcowfarm.com</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>older page shows info@)</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>.com email vs .com.au site. Some pages may be old.</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Two inboxes on contact page: hello@sculptedwax.com and sculptedwax@hotmail.com (</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1873,7 +1983,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>No Shopify evidence (/faqs URL not Shopify structure)</t>
+          <t>typo address on privacy page</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1916,7 +2026,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>321</v>
+        <v>363</v>
       </c>
     </row>
     <row r="3">
@@ -1926,7 +2036,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>323</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4">
@@ -1936,7 +2046,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>320</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE jewel/food/imp A rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>530</v>
+        <v>533</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E7" t="n">
         <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="G7" t="n">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kaffee / Specialty-Kaffeerösterei</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Taschen (Vintage Louis Vuitton)</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Taschen (Lederwaren, Rucksäcke, Geldbörsen)</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Feinkost (Öle, Senfe, RUB-Kräutermischungen, Geschenksets)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,10 +1435,40 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="B71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1478,7 +1508,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3">
@@ -1488,7 +1518,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4">
@@ -2026,7 +2056,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>363</v>
+        <v>365</v>
       </c>
     </row>
     <row r="3">
@@ -2036,7 +2066,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>365</v>
+        <v>367</v>
       </c>
     </row>
     <row r="4">
@@ -2046,7 +2076,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 14 complete: CA seeds, UK sweep, DE craft/kids + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>533</v>
+        <v>528</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>533</v>
+        <v>528</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>512</v>
+        <v>508</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="G3" t="n">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>69</v>
       </c>
       <c r="G4" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="G7" t="n">
-        <v>444</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="3">
@@ -1518,7 +1518,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4">
@@ -1983,7 +1983,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>Email from homepage only</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1993,7 +1993,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>Gmail-only inbox (rejected per batch rules).</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2003,17 +2003,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>Email seen in search summary but not tied to an exact snippet URL</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>typo address on privacy page</t>
+          <t>Email on wholesale subdomain</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2056,7 +2056,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3">
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>367</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4">
@@ -2076,7 +2076,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE imp C rows + hold; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E6" t="n">
         <v>4</v>
       </c>
       <c r="F6" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E7" t="n">
         <v>20</v>
       </c>
       <c r="F7" t="n">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="G7" t="n">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Feinkost (Öle, Senfe, RUB-Kräutermischungen, Geschenksets)</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,20 +1455,10 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
-        </is>
-      </c>
-      <c r="B71" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1518,7 +1508,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Round 15 UK/AU/CA sweeps + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>527</v>
+        <v>574</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>527</v>
+        <v>574</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>507</v>
+        <v>552</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>450</v>
+        <v>526</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="G2" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="G3" t="n">
-        <v>126</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="G4" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>73</v>
+        <v>87</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>69</v>
+        <v>83</v>
       </c>
       <c r="G5" t="n">
-        <v>111</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="G6" t="n">
-        <v>62</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>527</v>
+        <v>574</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>173</v>
+        <v>126</v>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
-        <v>507</v>
+        <v>552</v>
       </c>
       <c r="G7" t="n">
-        <v>450</v>
+        <v>526</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>55</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6">
@@ -819,37 +819,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Gift hampers &amp; corporate gift boxes</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Organic essential oils</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Handgefärbte Wolle &amp; Garne</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Hundezubehör &amp; Hundespielzeug</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Design-Zubehör für Hunde &amp; Katzen</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Personalisierte Kerzen, Kerzen-Bastelbedarf und Deko aus Dresden</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Natürliche Bartpflege (Bartöle, Bartbalsam, Bartseife, Rasieröl) aus Schleiden/Eifel</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,10 +1455,90 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
-      <c r="B70" t="n">
+      <c r="B78" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1498,7 +1578,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>231</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3">
@@ -1508,7 +1588,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4">
@@ -1518,7 +1598,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -1528,7 +1608,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -1538,7 +1618,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -1548,7 +1628,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -1558,7 +1638,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1617,7 +1697,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>125</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3">
@@ -1627,7 +1707,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>121</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4">
@@ -1637,7 +1717,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>100</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5">
@@ -1647,7 +1727,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>83</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6">
@@ -1657,7 +1737,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
@@ -1667,7 +1747,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -1683,21 +1763,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11">
@@ -1707,7 +1787,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -1717,7 +1797,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13">
@@ -1727,7 +1807,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14">
@@ -1737,7 +1817,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15">
@@ -1747,13 +1827,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>Email seen on homepage only</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -1763,27 +1843,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Email seen on homepage only</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1793,7 +1873,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1803,17 +1883,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>exact contact page not confirmed.</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1823,7 +1903,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Location not stated in results</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1833,37 +1913,37 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>exact contact page not confirmed.</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Email from homepage snippet only</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1873,7 +1953,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>no product detail or stated location found</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1883,7 +1963,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1893,7 +1973,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1903,7 +1983,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>Labelled decision-maker but role not stated</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1913,7 +1993,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1923,7 +2003,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>no specific product detail verified. Email not written.</t>
+          <t>no specific product detail verified.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1933,7 +2013,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>no product detail or stated location found</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1943,7 +2023,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Owner name inferred from brand name/inbox</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1953,7 +2033,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>resells other brands</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1963,7 +2043,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>confirm which to use.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1973,7 +2053,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Email from homepage only</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1983,7 +2063,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Gmail-only inbox (rejected per batch rules).</t>
+          <t>no specific product detail verified. Email not written.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1993,7 +2073,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not tied to an exact snippet URL</t>
+          <t>No product/collection detail verified</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2003,11 +2083,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Email on wholesale subdomain</t>
+          <t>No email found in search results</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2046,7 +2126,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>360</v>
+        <v>398</v>
       </c>
     </row>
     <row r="3">
@@ -2056,7 +2136,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>362</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4">
@@ -2066,7 +2146,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>359</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE seeds + home/beauty round 15, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>552</v>
+        <v>557</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>526</v>
+        <v>531</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="G6" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>552</v>
+        <v>557</v>
       </c>
       <c r="G7" t="n">
-        <v>526</v>
+        <v>531</v>
       </c>
     </row>
   </sheetData>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
@@ -825,31 +825,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Personalisierte Kerzen, Kerzen-Bastelbedarf und Deko aus Dresden</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Natürliche Bartpflege (Bartöle, Bartbalsam, Bartseife, Rasieröl) aus Schleiden/Eifel</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
+          <t>Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
+          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5">
@@ -1638,7 +1638,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -1648,7 +1648,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5">
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6">
@@ -1747,7 +1747,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="3">
@@ -2136,7 +2136,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
DE tech/gifts round 15 + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="G6" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E7" t="n">
         <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="G7" t="n">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
   </sheetData>
@@ -825,17 +825,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -845,7 +845,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -1578,7 +1578,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="3">
@@ -1598,7 +1598,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3">
@@ -2136,7 +2136,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4">
@@ -2146,7 +2146,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
UK round 16 sweeps + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>576</v>
+        <v>613</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>576</v>
+        <v>613</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>555</v>
+        <v>592</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>533</v>
+        <v>571</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>175</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10">
@@ -535,7 +535,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="G2" t="n">
-        <v>99</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
       </c>
       <c r="F3" t="n">
-        <v>107</v>
+        <v>122</v>
       </c>
       <c r="G3" t="n">
-        <v>140</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="G4" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E6" t="n">
         <v>5</v>
       </c>
       <c r="F6" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="G6" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>576</v>
+        <v>613</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>124</v>
+        <v>87</v>
       </c>
       <c r="E7" t="n">
         <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>555</v>
+        <v>592</v>
       </c>
       <c r="G7" t="n">
-        <v>533</v>
+        <v>571</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B78"/>
+  <dimension ref="A1:B90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -809,63 +809,63 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Automotive accessories</t>
+          <t>Kitchen and household products</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kitchen and household products</t>
+          <t>Automotive accessories</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Senf / Feinkost (handgemacht, Hamburg)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Hundehalsbänder &amp; Leinen (Leder, handgefertigt)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Hundehalsbänder &amp; Hundeleinen (Leder/BioThane, handgefertigt)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,10 +1535,130 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
           <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
-      <c r="B78" t="n">
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Quilting fabric, patterns &amp; supplies</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Quilting supplies &amp; longarm services</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Stationery &amp; paper goods</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1578,7 +1698,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>253</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3">
@@ -1588,7 +1708,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>116</v>
+        <v>129</v>
       </c>
     </row>
     <row r="4">
@@ -1598,7 +1718,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5">
@@ -1608,7 +1728,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -1618,7 +1738,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -1638,7 +1758,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1648,7 +1768,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -1697,7 +1817,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
@@ -1707,7 +1827,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
@@ -1717,7 +1837,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>136</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5">
@@ -1727,7 +1847,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6">
@@ -1737,7 +1857,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
@@ -1747,7 +1867,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -1767,7 +1887,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
     </row>
     <row r="10">
@@ -1787,7 +1907,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -1797,7 +1917,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13">
@@ -1807,7 +1927,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
@@ -1863,17 +1983,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1883,7 +2003,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1893,11 +2013,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>exact contact page not confirmed.</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -1907,23 +2027,23 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>Email from homepage only</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>exact contact page not confirmed.</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1933,7 +2053,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1943,27 +2063,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Email from homepage snippet only</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1973,7 +2093,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1983,7 +2103,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Labelled decision-maker but role not stated</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1993,7 +2113,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2003,7 +2123,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>no specific product detail verified.</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2013,7 +2133,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>no product detail or stated location found</t>
+          <t>Labelled decision-maker but role not stated</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2023,7 +2143,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2033,7 +2153,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>no specific product detail verified.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2043,7 +2163,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>confirm which to use.</t>
+          <t>no product detail or stated location found</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2053,7 +2173,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2063,7 +2183,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>no specific product detail verified. Email not written.</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2073,7 +2193,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>No product/collection detail verified</t>
+          <t>no product detail verified.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2083,7 +2203,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>No email found in search results</t>
+          <t>confirm which to use.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2126,7 +2246,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>399</v>
+        <v>433</v>
       </c>
     </row>
     <row r="3">
@@ -2136,7 +2256,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>401</v>
+        <v>435</v>
       </c>
     </row>
     <row r="4">
@@ -2146,7 +2266,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>398</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 16 CA/US/DE rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>613</v>
+        <v>628</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>613</v>
+        <v>628</v>
       </c>
     </row>
     <row r="5">
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>592</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>571</v>
+        <v>588</v>
       </c>
     </row>
     <row r="8">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>178</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="G2" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G4" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G6" t="n">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>613</v>
+        <v>628</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" t="n">
-        <v>592</v>
+        <v>606</v>
       </c>
       <c r="G7" t="n">
-        <v>571</v>
+        <v>588</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B90"/>
+  <dimension ref="A1:B94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
@@ -855,21 +855,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kitchen and household products</t>
+          <t>Automotive accessories</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Automotive accessories</t>
+          <t>Kitchen and household products</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -915,17 +915,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ceramics / tableware</t>
+          <t>Kaffeerösterei</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gift hampers &amp; corporate gift boxes</t>
+          <t>Ceramics / tableware</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Organic essential oils</t>
+          <t>Gift hampers &amp; corporate gift boxes</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Organic essential oils</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Handgefärbte Wolle &amp; Garne</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hundezubehör &amp; Hundespielzeug</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Design-Zubehör für Hunde &amp; Katzen</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Wolle &amp; Garne</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
+          <t>Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Senf / Feinkost (handgemacht, Hamburg)</t>
+          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
+          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Schokolade (Hamburg)</t>
+          <t>Hundezubehör / Lederhalsbänder</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Hundehalsbänder &amp; Leinen (Leder, handgefertigt)</t>
+          <t>Imkerei / Honig &amp; Geschenke</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hundehalsbänder &amp; Hundeleinen (Leder/BioThane, handgefertigt)</t>
+          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Kaffeerösterei / Kaffeealternativen</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Poster, Kunstdrucke, Postkarten</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Handmade fudge</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Beard care</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Personalised gifts</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Jigsaw puzzles</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Quilting fabric, patterns &amp; supplies</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Quilting supplies &amp; longarm services</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,10 +1655,50 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Quilting fabric, patterns &amp; supplies</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Quilting supplies &amp; longarm services</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
           <t>Stationery &amp; paper goods</t>
         </is>
       </c>
-      <c r="B90" t="n">
+      <c r="B94" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1698,7 +1738,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>262</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3">
@@ -1718,7 +1758,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -1728,7 +1768,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -1744,21 +1784,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Order status / fulfilment notifications</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Order status / fulfilment notifications</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -1768,7 +1808,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -1817,7 +1857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3">
@@ -1827,7 +1867,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -1837,7 +1877,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
@@ -1867,7 +1907,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8">
@@ -1963,7 +2003,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>confirm contact_source_url.</t>
+          <t>Email from homepage only</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -1973,17 +2013,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>no product detail verified</t>
+          <t>confirm contact_source_url.</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>no email written.</t>
+          <t>no product detail verified</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1993,17 +2033,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>no email written.</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -2013,7 +2053,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2023,7 +2063,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Location not stated in results</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2033,7 +2073,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Email from homepage only</t>
+          <t>Location not stated in results</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -2063,7 +2103,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2073,7 +2113,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2083,17 +2123,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>product detail generic.</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2103,7 +2143,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2113,7 +2153,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Email from homepage snippet only</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2123,7 +2163,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2133,7 +2173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Labelled decision-maker but role not stated</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2143,7 +2183,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>Labelled decision-maker but role not stated</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2153,7 +2193,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>no specific product detail verified.</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2163,7 +2203,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>no product detail or stated location found</t>
+          <t>no specific product detail verified.</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2173,7 +2213,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>no product detail or stated location found</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2183,7 +2223,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>Inbox domain differs from store domain</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2193,7 +2233,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>no product detail verified.</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2203,7 +2243,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>confirm which to use.</t>
+          <t>no product detail verified.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2246,7 +2286,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>433</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3">
@@ -2256,7 +2296,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>435</v>
+        <v>443</v>
       </c>
     </row>
     <row r="4">
@@ -2266,7 +2306,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>432</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US state B + DE coffee/honey rows, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>588</v>
+        <v>597</v>
       </c>
     </row>
     <row r="8">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="G2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="G3" t="n">
-        <v>157</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="G6" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7">
@@ -734,13 +734,13 @@
         <v>72</v>
       </c>
       <c r="E7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="G7" t="n">
-        <v>588</v>
+        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B94"/>
+  <dimension ref="A1:B93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="7">
@@ -915,17 +915,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kaffeerösterei</t>
+          <t>Ceramics / tableware</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ceramics / tableware</t>
+          <t>Gift hampers &amp; corporate gift boxes</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -935,7 +935,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Gift hampers &amp; corporate gift boxes</t>
+          <t>Organic essential oils</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Organic essential oils</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Handgefärbte Wolle &amp; Garne</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hundezubehör &amp; Hundespielzeug</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Design-Zubehör für Hunde &amp; Katzen</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
+          <t>Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Wolle &amp; Garne</t>
+          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
+          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
+          <t>Kaffeerösterei</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Kaffeerösterei / Kaffeealternativen</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Schokolade (Hamburg)</t>
+          <t>Poster, Kunstdrucke, Postkarten</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Poster, Kunstdrucke, Postkarten</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Handmade fudge</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Beard care</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Personalised gifts</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Jigsaw puzzles</t>
+          <t>Plant pots, planters and garden supplies</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1675,7 +1675,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Quilting fabric, patterns &amp; supplies</t>
+          <t>Quilting supplies &amp; longarm services</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1685,20 +1685,10 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Quilting supplies &amp; longarm services</t>
+          <t>Stationery &amp; paper goods</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>Stationery &amp; paper goods</t>
-        </is>
-      </c>
-      <c r="B94" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1748,7 +1738,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4">
@@ -1758,7 +1748,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -1778,7 +1768,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -1798,7 +1788,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -1808,7 +1798,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -2233,7 +2223,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>verify contact page before sending.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2243,7 +2233,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>no product detail verified.</t>
+          <t>Shopify proof is URL structure only.</t>
         </is>
       </c>
       <c r="B41" t="n">

</xml_diff>

<commit_message>
DE sweep C, CA sweep D, UK home rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>628</v>
+        <v>620</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>628</v>
+        <v>620</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>605</v>
+        <v>597</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>597</v>
+        <v>605</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" t="n">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="G4" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G6" t="n">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>628</v>
+        <v>620</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
+        <v>597</v>
+      </c>
+      <c r="G7" t="n">
         <v>605</v>
-      </c>
-      <c r="G7" t="n">
-        <v>597</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B93"/>
+  <dimension ref="A1:B91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5">
@@ -819,23 +819,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -849,7 +849,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Poster, Kunstdrucke, Postkarten</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Handmade fudge</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Beard care</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Personalised gifts</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Jigsaw puzzles</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Plant pots, planters and garden supplies</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,7 +1655,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Quilting supplies &amp; longarm services</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1665,30 +1665,10 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Stationery &amp; paper goods</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>Quilting supplies &amp; longarm services</t>
-        </is>
-      </c>
-      <c r="B92" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>Stationery &amp; paper goods</t>
-        </is>
-      </c>
-      <c r="B93" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1728,7 +1708,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3">
@@ -1748,7 +1728,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -1758,7 +1738,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6">
@@ -1983,17 +1963,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Email seen on homepage only</t>
+          <t>Email from homepage only</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Email from homepage only</t>
+          <t>Email seen on homepage only</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2233,7 +2213,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Shopify proof is URL structure only.</t>
+          <t>Mixed URL patterns</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2276,7 +2256,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>441</v>
+        <v>434</v>
       </c>
     </row>
     <row r="3">
@@ -2286,7 +2266,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>443</v>
+        <v>436</v>
       </c>
     </row>
     <row r="4">
@@ -2296,7 +2276,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>440</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
AU sweep F round 16 + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>620</v>
+        <v>631</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>620</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>597</v>
+        <v>608</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>605</v>
+        <v>620</v>
       </c>
     </row>
     <row r="8">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="G4" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G5" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>620</v>
+        <v>631</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>80</v>
+        <v>69</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="G7" t="n">
-        <v>605</v>
+        <v>620</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -815,21 +815,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8">
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="3">
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
@@ -1764,7 +1764,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1774,11 +1774,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10">
@@ -2013,17 +2013,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Gmail inbox only</t>
+          <t>no specific product verified.</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>no email drafted.</t>
+          <t>Gmail inbox only</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2033,7 +2033,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>no specific product verified.</t>
+          <t>no email drafted.</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -2073,7 +2073,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>confirm main inbox.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2083,7 +2083,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2093,7 +2093,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2103,17 +2103,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>product detail generic.</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2123,7 +2123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2133,7 +2133,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Email from homepage snippet only</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2143,7 +2143,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2153,7 +2153,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Labelled decision-maker but role not stated</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2163,7 +2163,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>multi-brand retailer.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2173,7 +2173,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>no specific product detail verified.</t>
+          <t>Labelled decision-maker but role not stated</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2183,7 +2183,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>no product detail or stated location found</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2193,7 +2193,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Inbox domain differs from store domain</t>
+          <t>no specific product detail verified.</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2203,7 +2203,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>verify contact page before sending.</t>
+          <t>no named product.</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2213,7 +2213,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mixed URL patterns</t>
+          <t>no product detail or stated location found</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>434</v>
+        <v>445</v>
       </c>
     </row>
     <row r="3">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>436</v>
+        <v>447</v>
       </c>
     </row>
     <row r="4">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>433</v>
+        <v>444</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 16 complete: CA sweep C + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>608</v>
+        <v>606</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
     <row r="8">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G4" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="G7" t="n">
-        <v>620</v>
+        <v>622</v>
       </c>
     </row>
   </sheetData>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3">
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
@@ -1764,7 +1764,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pre-order / launch / drop stock management</t>
+          <t>Multi-location / multi-channel sync</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1774,11 +1774,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Multi-location / multi-channel sync</t>
+          <t>Pre-order / launch / drop stock management</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -2203,7 +2203,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>no named product.</t>
+          <t>Location from search summary only</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2213,7 +2213,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>no product detail or stated location found</t>
+          <t>no named product.</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2256,7 +2256,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>445</v>
+        <v>443</v>
       </c>
     </row>
     <row r="3">
@@ -2266,7 +2266,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>447</v>
+        <v>445</v>
       </c>
     </row>
     <row r="4">
@@ -2276,7 +2276,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US food + UK beauty/home round 17, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>629</v>
+        <v>660</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>629</v>
+        <v>660</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>606</v>
+        <v>637</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>622</v>
+        <v>646</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="G2" t="n">
-        <v>114</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="G3" t="n">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="G4" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="G6" t="n">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>629</v>
+        <v>660</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>606</v>
+        <v>637</v>
       </c>
       <c r="G7" t="n">
-        <v>622</v>
+        <v>646</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B91"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4">
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -809,47 +809,47 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Fitness and sports equipment</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Fitness and sports equipment</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Handmade ceramics (paint palettes, mugs, garden markers)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Handcrafted wood cutting boards, charcuterie boards and custom tables</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Handgefärbte Wolle &amp; Garne</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hundezubehör &amp; Hundespielzeug</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Design-Zubehör für Hunde &amp; Katzen</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Wolle &amp; Garne</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
+          <t>Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Kaffeerösterei</t>
+          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hundezubehör / Lederhalsbänder</t>
+          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Imkerei / Honig &amp; Geschenke</t>
+          <t>Kaffeerösterei</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
+          <t>Hundezubehör / Lederhalsbänder</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
+          <t>Imkerei / Honig &amp; Geschenke</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Schokolade (Hamburg)</t>
+          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Honig / Imkereiprodukte</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Tee &amp; Matcha-Zubehör</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Tee</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Handmade fudge</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Beard care</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Personalised gifts</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jigsaw puzzles</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Handmade stoneware planters and ceramics</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Handmade animal-themed ceramics and planters</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Board games and tabletop games (shops in Cardiff and Bristol)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,7 +1655,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Quilting supplies &amp; longarm services</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1665,10 +1665,100 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Handmade leather camera straps</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Essential oils and aromatherapy</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Quilting supplies &amp; longarm services</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>Stationery &amp; paper goods</t>
         </is>
       </c>
-      <c r="B91" t="n">
+      <c r="B100" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1708,7 +1798,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3">
@@ -1718,7 +1808,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>128</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4">
@@ -1728,7 +1818,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
@@ -1738,7 +1828,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -1748,7 +1838,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -1758,7 +1848,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -1768,7 +1858,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1778,7 +1868,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -1827,7 +1917,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3">
@@ -1837,7 +1927,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4">
@@ -1847,7 +1937,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5">
@@ -1857,7 +1947,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6">
@@ -1867,7 +1957,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7">
@@ -1877,13 +1967,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>no valid email</t>
+          <t>Shopify not verified</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1893,11 +1983,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shopify not verified</t>
+          <t>no valid email</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
@@ -1937,7 +2027,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14">
@@ -2063,7 +2153,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>Email from homepage snippet only</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -2073,7 +2163,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>confirm main inbox.</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2083,7 +2173,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>confirm main inbox.</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2093,7 +2183,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2103,7 +2193,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2113,17 +2203,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>product detail generic.</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2133,7 +2223,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2143,7 +2233,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email from homepage snippet only</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2256,7 +2346,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>443</v>
+        <v>469</v>
       </c>
     </row>
     <row r="3">
@@ -2266,7 +2356,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>445</v>
+        <v>471</v>
       </c>
     </row>
     <row r="4">
@@ -2276,7 +2366,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>442</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US quilt/pet + DE sweep D round 17, holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>660</v>
+        <v>674</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>660</v>
+        <v>674</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>637</v>
+        <v>651</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>646</v>
+        <v>688</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C2" t="n">
         <v>250</v>
       </c>
       <c r="D2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E2" t="n">
         <v>7</v>
       </c>
       <c r="F2" t="n">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G2" t="n">
-        <v>122</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G3" t="n">
-        <v>167</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C4" t="n">
         <v>100</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="G4" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="G5" t="n">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6">
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G6" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>660</v>
+        <v>674</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>637</v>
+        <v>651</v>
       </c>
       <c r="G7" t="n">
-        <v>646</v>
+        <v>688</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B100"/>
+  <dimension ref="A1:B104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -779,7 +779,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4">
@@ -809,37 +809,37 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Home decor and furniture</t>
+          <t>Pet products and accessories</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Baby and children's products</t>
+          <t>Home decor and furniture</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pet products and accessories</t>
+          <t>Baby and children's products</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9">
@@ -945,7 +945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Handmade designer cushions, lampshades and upholstery</t>
+          <t>Saddlery / equestrian</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -955,7 +955,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Stationery, notebooks and writing instruments</t>
+          <t>Handmade designer cushions, lampshades and upholstery</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -965,7 +965,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Handmade ceramics (paint palettes, mugs, garden markers)</t>
+          <t>Stationery, notebooks and writing instruments</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -975,7 +975,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Handcrafted wood cutting boards, charcuterie boards and custom tables</t>
+          <t>Handmade ceramics (paint palettes, mugs, garden markers)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -985,7 +985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Waterproof leather winter boots</t>
+          <t>Handcrafted wood cutting boards, charcuterie boards and custom tables</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -995,7 +995,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Hundefutter (BARF &amp; Nassfutter)</t>
+          <t>Waterproof leather winter boots</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1005,7 +1005,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Handgemachte Schneidebretter aus Holz</t>
+          <t>Hundefutter (BARF &amp; Nassfutter)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1015,7 +1015,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör</t>
+          <t>Handgemachte Schneidebretter aus Holz</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1025,7 +1025,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
+          <t>Handgemachtes Hundezubehör</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1035,7 +1035,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Handgefärbte Wolle &amp; Garne</t>
+          <t>Handgemachte Hundeleinen &amp; Halsbänder</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1045,7 +1045,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
+          <t>Handgefärbte Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1055,7 +1055,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tee / Teemischungen</t>
+          <t>Handgefertigtes Katzenspielzeug, Schlafplätze &amp; Kratzmöbel</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1065,7 +1065,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Vegane Duftkerzen aus Sojawachs</t>
+          <t>Tee / Teemischungen</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1075,7 +1075,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
+          <t>Vegane Duftkerzen aus Sojawachs</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1085,7 +1085,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
+          <t>Personalisierte Geschenke (Stoffbeutel, Keramik-Spardosen)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1095,7 +1095,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Hundezubehör &amp; Hundespielzeug</t>
+          <t>Handgemachtes Hundezubehör (BioThane &amp; Leder)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1105,7 +1105,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Design-Zubehör für Hunde &amp; Katzen</t>
+          <t>Hundezubehör &amp; Hundespielzeug</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1115,7 +1115,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
+          <t>Design-Zubehör für Hunde &amp; Katzen</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1125,7 +1125,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
+          <t>Handgemachte Stirnholz-Schneidebretter (Küche)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1135,7 +1135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
+          <t>Alkoholfreie Kräuter-Aperitifs / Spritz</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1145,7 +1145,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
+          <t>Handgefertigte Massivholzmöbel (Schreibtische, Sideboards) aus Dresden</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1155,7 +1155,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
+          <t>Lederwaren Made in Germany (Kleinlederwaren, Taschen)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1165,7 +1165,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
+          <t>Ledergürtel &amp; Lederaccessoires, handgemacht in Berlin</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1175,7 +1175,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Wolle &amp; Garne</t>
+          <t>Holz-Lernspiele für Kinder (Lochkasten / Puncho)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1185,7 +1185,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
+          <t>Wolle &amp; Garne</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -1195,7 +1195,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
+          <t>Personalisierte Geschenke (Lasergravur &amp; Stickerei)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -1205,7 +1205,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Kaffeerösterei</t>
+          <t>Kaffeerösterei / Espresso &amp; Filterkaffee</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1215,7 +1215,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Hundezubehör / Lederhalsbänder</t>
+          <t>Kaffeerösterei</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1225,7 +1225,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Imkerei / Honig &amp; Geschenke</t>
+          <t>Hundezubehör / Lederhalsbänder</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1235,7 +1235,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
+          <t>Imkerei / Honig &amp; Geschenke</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
+          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Schokolade (Hamburg)</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Honig / Imkereiprodukte</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Board games and tabletop games (shops in Cardiff and Bristol)</t>
+          <t>Letterbox iced biscuit gifts</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Artisan cheese gift boxes</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Board games and tabletop games (shops in Cardiff and Bristol)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Letterpress greeting cards &amp; stationery</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Letterpress stationery, bookbinding &amp; gifts</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,7 +1655,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1665,7 +1665,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1675,7 +1675,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1685,7 +1685,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1695,7 +1695,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1705,7 +1705,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1715,7 +1715,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1725,7 +1725,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1735,7 +1735,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1745,7 +1745,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Quilting supplies &amp; longarm services</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1755,10 +1755,50 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Quilting supplies &amp; longarm services</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>Stationery &amp; paper goods</t>
         </is>
       </c>
-      <c r="B100" t="n">
+      <c r="B104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1798,7 +1838,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>277</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3">
@@ -1838,7 +1878,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7">
@@ -1848,7 +1888,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -1858,7 +1898,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -1868,7 +1908,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10">
@@ -1917,7 +1957,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>173</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3">
@@ -1927,7 +1967,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>170</v>
+        <v>184</v>
       </c>
     </row>
     <row r="4">
@@ -1937,7 +1977,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>151</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5">
@@ -1947,7 +1987,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>127</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6">
@@ -1957,7 +1997,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -1967,7 +2007,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -1977,7 +2017,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -1993,21 +2033,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>no contact source URL</t>
+          <t>email body N words (need 75–120)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>email body N words (need 75–120)</t>
+          <t>no contact source URL</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
@@ -2017,7 +2057,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -2027,7 +2067,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -2037,7 +2077,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
@@ -2047,7 +2087,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -2163,7 +2203,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Email domain differs from store domain</t>
+          <t>multi-brand retailer.</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -2173,7 +2213,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>confirm main inbox.</t>
+          <t>Email domain differs from store domain</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -2183,7 +2223,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>confirm main inbox.</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2193,7 +2233,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>no product detail verified. Email not written.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2203,7 +2243,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>No product/collection detail verified</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2213,37 +2253,37 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>product detail generic.</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -2253,7 +2293,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>multi-brand retailer.</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -2263,7 +2303,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Labelled decision-maker but role not stated</t>
+          <t>several inboxes</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2273,7 +2313,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2283,7 +2323,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>no specific product detail verified.</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2293,7 +2333,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Location from search summary only</t>
+          <t>Labelled decision-maker but role not stated</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2303,7 +2343,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>no named product.</t>
+          <t>Multi-brand boutique</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2346,7 +2386,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>469</v>
+        <v>484</v>
       </c>
     </row>
     <row r="3">
@@ -2356,7 +2396,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>471</v>
+        <v>486</v>
       </c>
     </row>
     <row r="4">
@@ -2366,7 +2406,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>468</v>
+        <v>483</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 17 UK/CA/US rows + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>688</v>
+        <v>691</v>
       </c>
     </row>
     <row r="8">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C3" t="n">
         <v>150</v>
       </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
         <v>5</v>
       </c>
       <c r="F3" t="n">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G3" t="n">
-        <v>179</v>
+        <v>182</v>
       </c>
     </row>
     <row r="4">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="G7" t="n">
-        <v>688</v>
+        <v>691</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B104"/>
+  <dimension ref="A1:B102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Artisan cheese gift boxes</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Board games and tabletop games (shops in Cardiff and Bristol)</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Letterpress greeting cards &amp; stationery</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
+          <t>Letterpress stationery, bookbinding &amp; gifts</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Letterpress greeting cards &amp; stationery</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Letterpress stationery, bookbinding &amp; gifts</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,7 +1655,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1665,7 +1665,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1675,7 +1675,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1685,7 +1685,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1695,7 +1695,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1705,7 +1705,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1715,7 +1715,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1725,7 +1725,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1735,7 +1735,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1745,7 +1745,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1755,7 +1755,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1765,7 +1765,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Quilting supplies &amp; longarm services</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1775,30 +1775,10 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Stationery &amp; paper goods</t>
         </is>
       </c>
       <c r="B102" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Quilting supplies &amp; longarm services</t>
-        </is>
-      </c>
-      <c r="B103" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
-        <is>
-          <t>Stationery &amp; paper goods</t>
-        </is>
-      </c>
-      <c r="B104" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1848,7 +1828,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4">
@@ -1868,7 +1848,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
@@ -1908,7 +1888,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
@@ -2097,7 +2077,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -2223,7 +2203,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>confirm main inbox.</t>
+          <t>Mixed URL patterns</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -2233,7 +2213,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>no product detail verified. Email not written.</t>
+          <t>confirm main inbox.</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -2243,7 +2223,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>No product/collection detail verified</t>
+          <t>no product detail verified. Email not written.</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -2253,7 +2233,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>email on product page</t>
+          <t>No product/collection detail verified</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -2263,7 +2243,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Email seen in search summary but not quoted on the cited page</t>
+          <t>email on product page</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -2273,7 +2253,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>No public email found</t>
+          <t>possibly mid-size</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -2283,27 +2263,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>No specific product/collection verified</t>
+          <t>Email seen in search summary but not quoted on the cited page</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>product detail generic.</t>
+          <t>No public email found</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>several inboxes</t>
+          <t>No specific product/collection verified</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -2313,7 +2293,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Email on homepage</t>
+          <t>product detail generic.</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -2323,7 +2303,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>No specific product/collection detail verified</t>
+          <t>several inboxes</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -2333,7 +2313,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Labelled decision-maker but role not stated</t>
+          <t>Email on homepage</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -2343,7 +2323,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Multi-brand boutique</t>
+          <t>No specific product/collection detail verified</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -2386,7 +2366,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="3">
@@ -2396,7 +2376,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="4">
@@ -2406,7 +2386,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round 17 complete: AU sweep G + holds; rebuild
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
     <row r="8">
@@ -675,22 +675,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C5" t="n">
         <v>100</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
         <v>4</v>
       </c>
       <c r="F5" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G5" t="n">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="G7" t="n">
-        <v>691</v>
+        <v>694</v>
       </c>
     </row>
   </sheetData>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4">
@@ -819,7 +819,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3">
@@ -1858,7 +1858,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -1878,7 +1878,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -2366,7 +2366,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="3">
@@ -2376,7 +2376,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>483</v>
+        <v>480</v>
       </c>
     </row>
     <row r="4">
@@ -2386,7 +2386,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finish outreach day 3; hold two leads with outdated observations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R5gXYQek1J6Kb2P6BuuFjU
</commit_message>
<xml_diff>
--- a/shopify-leads/Shopify_Research_Summary.xlsx
+++ b/shopify-leads/Shopify_Research_Summary.xlsx
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="5">
@@ -494,7 +494,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="7">
@@ -504,7 +504,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
     <row r="8">
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10">
@@ -535,7 +535,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -700,22 +700,22 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C6" t="n">
         <v>100</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
         <v>6</v>
       </c>
       <c r="F6" t="n">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G6" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7">
@@ -725,22 +725,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="C7" t="n">
         <v>700</v>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
       </c>
       <c r="F7" t="n">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="G7" t="n">
-        <v>694</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -795,17 +795,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Jewelry and accessories</t>
+          <t>Skincare and beauty products</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Skincare and beauty products</t>
+          <t>Jewelry and accessories</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1245,7 +1245,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Imkerei / Honig &amp; Bienenpatenschaften</t>
+          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1255,7 +1255,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Logo-Schokolade, Pralinen, Firmenpräsente</t>
+          <t>Schokolade (Hamburg)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -1265,7 +1265,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Schokolade (Hamburg)</t>
+          <t>Tee &amp; Matcha-Zubehör</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -1275,7 +1275,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tee &amp; Matcha-Zubehör</t>
+          <t>Tee</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -1285,7 +1285,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Tee</t>
+          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1295,7 +1295,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Handgemachte Naturseifen (Seifenmanufaktur)</t>
+          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1305,7 +1305,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Taschen und Lederwaren aus sämisch gegerbtem Hirschleder</t>
+          <t>Wolle / Garn / Bastelbedarf</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1315,7 +1315,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Wolle / Garn / Bastelbedarf</t>
+          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1325,7 +1325,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Specialty-Kaffeerösterei (Espresso, Filterkaffee, Zubehör)</t>
+          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1335,7 +1335,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Kaffeerösterei (Espresso, Filterkaffee, Kaffee-Abo)</t>
+          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1345,7 +1345,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bio-Schokolade und Pralinen ohne Industriezucker</t>
+          <t>Handgefertigte Bio-Schokoladentafeln</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1355,7 +1355,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Handgefertigte Bio-Schokoladentafeln</t>
+          <t>Loser Premium-Tee und Zubehör</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1365,7 +1365,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Loser Premium-Tee und Zubehör</t>
+          <t>Handgefertigtes Hundezubehör</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1375,7 +1375,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Handgefertigtes Hundezubehör</t>
+          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1385,7 +1385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Tiefkühlkost &amp; Lebensmittel (Pelmeni, Brot) — off assigned niche</t>
+          <t>Stationery / notebooks / fountain pen ink</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1395,7 +1395,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Stationery / notebooks / fountain pen ink</t>
+          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1405,7 +1405,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Jams, chutneys and relishes (Mevagissey, Cornwall)</t>
+          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1415,7 +1415,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Needlework craft kits (tapestry, needlepoint, cross stitch, embroidery)</t>
+          <t>Handmade fudge</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1425,7 +1425,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Handmade fudge</t>
+          <t>Beard care</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1435,7 +1435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Beard care</t>
+          <t>Personalised gifts</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1445,7 +1445,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Personalised gifts</t>
+          <t>Jigsaw puzzles</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1455,7 +1455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Jigsaw puzzles</t>
+          <t>Handmade stoneware planters and ceramics</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1465,7 +1465,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Handmade stoneware planters and ceramics</t>
+          <t>Handmade animal-themed ceramics and planters</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1475,7 +1475,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Handmade animal-themed ceramics and planters</t>
+          <t>Letterbox iced biscuit gifts</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1485,7 +1485,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Letterbox iced biscuit gifts</t>
+          <t>Natural plastic-free deodorant and body care</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1495,7 +1495,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Natural plastic-free deodorant and body care</t>
+          <t>Natural bath &amp; body products (refills, gift sets)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1505,7 +1505,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Natural bath &amp; body products (refills, gift sets)</t>
+          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1515,7 +1515,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Handmade fruit preserves, jams and marmalades (Pacifica, CA)</t>
+          <t>Letterpress greeting cards &amp; stationery</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1525,7 +1525,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Letterpress greeting cards &amp; stationery</t>
+          <t>Letterpress stationery, bookbinding &amp; gifts</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1535,7 +1535,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Letterpress stationery, bookbinding &amp; gifts</t>
+          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1545,7 +1545,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Handmade leather belts, wallets and small goods (Deer Park, WA)</t>
+          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1555,7 +1555,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Biodegradable body wash and bath products (San Francisco, CA)</t>
+          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1565,7 +1565,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Black-owned small-batch whipped body butters, creams and body oils (NYC)</t>
+          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -1575,7 +1575,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Stationery (fountain pens, inks, notebooks; Chicago, IL store + online)</t>
+          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1585,7 +1585,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Stationery and gifts (planners, journals, gift bundles; Southern California)</t>
+          <t>Organic and heirloom garden seeds and seed kits</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1595,7 +1595,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Organic and heirloom garden seeds and seed kits</t>
+          <t>Culturally important open-pollinated seeds from small farms</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1605,7 +1605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Culturally important open-pollinated seeds from small farms</t>
+          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1615,7 +1615,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Non-GMO, open-pollinated vegetable, herb and flower seeds</t>
+          <t>Designer colored glassware and tableware</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1625,7 +1625,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Designer colored glassware and tableware</t>
+          <t>Pickleball paddles and accessories</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -1635,7 +1635,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Pickleball paddles and accessories</t>
+          <t>Pickleball paddles and gear</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1645,7 +1645,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Pickleball paddles and gear</t>
+          <t>Handmade leather golf headcovers</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1655,7 +1655,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Handmade leather golf headcovers</t>
+          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1665,7 +1665,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Mechanical keyboards, keycaps &amp; deskpads</t>
+          <t>Custom mechanical keyboards &amp; keycaps</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1675,7 +1675,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Custom mechanical keyboards &amp; keycaps</t>
+          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1685,7 +1685,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Custom keyboards, EC conversion kits &amp; PCBs</t>
+          <t>Handmade leather camera straps</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1695,7 +1695,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Handmade leather camera straps</t>
+          <t>Essential oils and aromatherapy</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1705,7 +1705,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Essential oils and aromatherapy</t>
+          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -1715,7 +1715,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Stationery: fountain pen ink, fountain pens, washi tape, stickers, sticky notes</t>
+          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1725,7 +1725,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Small-batch jams, jellies, pickles and farm eggs (Floresville, TX)</t>
+          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -1735,7 +1735,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Independent yarn, fabric and craft store (Northeast Minneapolis, MN)</t>
+          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1745,7 +1745,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Hand-dyed yarns for knitters, crocheters and weavers (Mountain City, TN)</t>
+          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1755,7 +1755,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Quilt shop, natural fiber fabric and longarm quilting (Cleveland, Tennessee)</t>
+          <t>Quilting supplies &amp; longarm services</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1765,20 +1765,10 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Quilting supplies &amp; longarm services</t>
+          <t>Stationery &amp; paper goods</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
-        <is>
-          <t>Stationery &amp; paper goods</t>
-        </is>
-      </c>
-      <c r="B102" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1818,7 +1808,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3">
@@ -1868,7 +1858,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">

</xml_diff>